<commit_message>
redundancy.py: wait = catch the same bus N days later, router free to substitute; rerun results
Leaf script, nothing imports it (regress not rerun).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/redundancy.xlsx
+++ b/docs/redundancy.xlsx
@@ -759,11 +759,11 @@
         </is>
       </c>
       <c r="E12" s="2" t="n">
-        <v>144</v>
+        <v>24</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>d11 Sat 18:33 Omnitrans: Vine Street Mobility Hub -&gt; San Bernardino Transit Center</t>
+          <t>wait 1 day(s) and catch the same bus, then continue</t>
         </is>
       </c>
     </row>
@@ -899,11 +899,11 @@
         </is>
       </c>
       <c r="E17" s="2" t="n">
-        <v>96</v>
+        <v>24</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>d13 Mon 22:00 Greyhound-us: Houston Bus Station (Greyhound) -&gt; Mobile Bus Station</t>
+          <t>wait 1 day(s) and catch the same bus, then continue</t>
         </is>
       </c>
     </row>
@@ -927,11 +927,11 @@
         </is>
       </c>
       <c r="E18" s="2" t="n">
-        <v>81.40000000000001</v>
+        <v>24</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>d14 Tue 17:10 Greyhound-us: Tallahassee (CK Steele Bus Plaza) -&gt; Jacksonville (Downtown)</t>
+          <t>wait 1 day(s) and catch the same bus, then continue</t>
         </is>
       </c>
     </row>
@@ -1011,11 +1011,11 @@
         </is>
       </c>
       <c r="E21" s="2" t="n">
-        <v>81.40000000000001</v>
+        <v>24</v>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>d15 Wed 07:10 Amtrak: Washington Union Station -&gt; Stamford Amtrak Station</t>
+          <t>wait 1 day(s) and catch the same bus, then continue</t>
         </is>
       </c>
     </row>
@@ -1039,11 +1039,11 @@
         </is>
       </c>
       <c r="E22" s="2" t="n">
-        <v>57.4</v>
+        <v>24</v>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>d15 Wed 15:30 Dartmouth Coach: Boston South Station -&gt; Hanover (Hanover Inn)</t>
+          <t>wait 1 day(s) and catch the same bus, then continue</t>
         </is>
       </c>
     </row>
@@ -1067,11 +1067,11 @@
         </is>
       </c>
       <c r="E23" s="2" t="n">
-        <v>57.4</v>
+        <v>24</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>d15 Wed 17:23 Advance Transit: Hanover Inn -&gt; Vail DMS</t>
+          <t>wait 1 day(s) and catch the same bus, then continue</t>
         </is>
       </c>
     </row>
@@ -1772,11 +1772,11 @@
         </is>
       </c>
       <c r="E3" s="2" t="n">
-        <v>117.5</v>
+        <v>24</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>d9 Thu 03:30 Greyhound-us: Huntington Bus Stop -&gt; Beckley Intermodal Parking Garage</t>
+          <t>wait 1 day(s) and catch the same bus, then continue</t>
         </is>
       </c>
     </row>
@@ -1800,11 +1800,11 @@
         </is>
       </c>
       <c r="E4" s="2" t="n">
-        <v>117.5</v>
+        <v>24</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>d9 Thu 07:30 Greyhound-us: Columbus Bus Station -&gt; Cleveland (E 12th St)</t>
+          <t>wait 1 day(s) and catch the same bus, then continue</t>
         </is>
       </c>
     </row>
@@ -1828,11 +1828,11 @@
         </is>
       </c>
       <c r="E5" s="2" t="n">
-        <v>117.5</v>
+        <v>24</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>d9 Thu 17:05 Barons Bus Lines: Detroit -&gt; Indianapolis</t>
+          <t>wait 1 day(s) and catch the same bus, then continue</t>
         </is>
       </c>
     </row>
@@ -1856,11 +1856,11 @@
         </is>
       </c>
       <c r="E6" s="2" t="n">
-        <v>117.5</v>
+        <v>24</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>d9 Thu 20:05 Greyhound-us: Indianapolis Bus Station -&gt; Dayton Trotwood Bus Station</t>
+          <t>wait 1 day(s) and catch the same bus, then continue</t>
         </is>
       </c>
     </row>
@@ -2192,11 +2192,11 @@
         </is>
       </c>
       <c r="E18" s="2" t="n">
-        <v>92.5</v>
+        <v>24</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>d12 Sun 07:10 Greyhound-us: Eau Claire (McDonald's) -&gt; Minneapolis Bus Station</t>
+          <t>wait 1 day(s) and catch the same bus, then continue</t>
         </is>
       </c>
     </row>
@@ -2220,11 +2220,11 @@
         </is>
       </c>
       <c r="E19" s="2" t="n">
-        <v>92.5</v>
+        <v>24</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>d12 Sun 10:35 Jefferson Lines: Minneapolis -&gt; Billings</t>
+          <t>wait 1 day(s) and catch the same bus, then continue</t>
         </is>
       </c>
     </row>
@@ -2416,11 +2416,11 @@
         </is>
       </c>
       <c r="E26" s="2" t="n">
-        <v>92.5</v>
+        <v>24</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>d14 Tue 18:55 Greyhound-us: San Bernardino Depot -&gt; Las Vegas Bus Terminal</t>
+          <t>wait 1 day(s) and catch the same bus, then continue</t>
         </is>
       </c>
     </row>
@@ -2957,7 +2957,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>wait 1 day(s): the same buses run, everything shifts</t>
+          <t>wait 1 day(s) and catch the same bus, then continue</t>
         </is>
       </c>
     </row>
@@ -3041,7 +3041,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>wait 1 day(s): the same buses run, everything shifts</t>
+          <t>wait 1 day(s) and catch the same bus, then continue</t>
         </is>
       </c>
     </row>
@@ -3069,7 +3069,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>wait 1 day(s): the same buses run, everything shifts</t>
+          <t>wait 1 day(s) and catch the same bus, then continue</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
redundancy: clean four-route run (one process); X's Chief miss +24 h
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/redundancy.xlsx
+++ b/docs/redundancy.xlsx
@@ -8,8 +8,9 @@
   </bookViews>
   <sheets>
     <sheet name="X" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Control" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Record" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Moorhead" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Control" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Record" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1702,6 +1703,1159 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:F41"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="4" customWidth="1" min="1" max="1"/>
+    <col width="36" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="100" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Moorhead: 250.26 h. Miss each ride by one minute and replay the rest.</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>missed</t>
+        </is>
+      </c>
+      <c r="C2" s="1" t="inlineStr">
+        <is>
+          <t>from</t>
+        </is>
+      </c>
+      <c r="D2" s="1" t="inlineStr">
+        <is>
+          <t>to</t>
+        </is>
+      </c>
+      <c r="E2" s="1" t="inlineStr">
+        <is>
+          <t>cost h</t>
+        </is>
+      </c>
+      <c r="F2" s="1" t="inlineStr">
+        <is>
+          <t>recovery starts with</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>d1 Mon 14:30 Jefferson Lines</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Fargo</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Sioux Falls</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>d1 Mon 16:40 Jefferson Lines: Fargo -&gt; Minneapolis</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>2</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>d1 Mon 19:00 Jefferson Lines</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Sioux Falls</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Maryville</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>d2 Tue 19:00 Jefferson Lines: Sioux Falls -&gt; Maryville</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>3</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>d2 Tue 03:25 Jefferson Lines</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Maryville</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Omaha</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>d3 Wed 03:25 Jefferson Lines: Maryville -&gt; Omaha</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>4</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>d2 Tue 06:15 Jefferson Lines</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Omaha</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Sioux Falls</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>d3 Wed 06:15 Jefferson Lines: Omaha -&gt; Sioux Falls</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>5</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>d2 Tue 12:40 Jefferson Lines</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Sioux Falls</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Billings</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>d2 Tue 18:45 Jefferson Lines: Sioux Falls -&gt; Minneapolis</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>6</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>d3 Wed 01:30 Jefferson Lines</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Billings</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Spokane</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>d4 Thu 01:30 Jefferson Lines: Billings -&gt; Spokane</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>7</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>d3 Wed 10:45 Northwestern Stage Lines</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Spokane</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Pasco Bus Stop</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>d3 Wed 11:10 FlixBus-us: Spokane Station -&gt; Pasco Bus Stop</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>8</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>d3 Wed 13:25 Greyhound-us</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Pasco Bus Stop</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Salt Lake City Intermodal Trans Ctr</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>d3 Wed 15:00 Northwestern Stage Lines: Pasco Bus Stop -&gt; Boise (Airport)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>9</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>d4 Thu 04:45 Salt Lake Express</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Salt Lake City (Airport)</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Saint George (Bluff St Office)</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>d4 Thu 06:00 Salt Lake Express: Salt Lake City (Airport) -&gt; Las Vegas (Airport)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>10</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>d4 Thu 10:30 Salt Lake Express</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Saint George (Bluff St Office)</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Las Vegas (Airport)</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>d4 Thu 12:00 Salt Lake Express: Saint George (Bluff St Office) -&gt; Las Vegas (Airport)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>11</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>d4 Thu 14:00 Greyhound-us</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Las Vegas Bus Terminal</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>San Bernardino Depot</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>d4 Thu 15:15 702 Shuttles: Las Vegas Dean Martin Blue Diamond (702 Shuttles) -&gt; Victorville 15445 Palmdale Rd (702 Shuttles)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>12</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>d4 Thu 18:43 Amtrak</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>San Bernardino</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Newton</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="n">
+        <v>144</v>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>d4 Thu 18:55 Greyhound-us: San Bernardino Depot -&gt; Las Vegas Bus Terminal</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>13</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>d6 Sat 03:00 BeeLine Express-Village Travel</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Newton (Amtrak)</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Oklahoma City</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>d6 Sat 04:00 Beeline Express: Newton -&gt; Oklahoma City</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>14</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>d6 Sat 06:55 Greyhound-us</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Oklahoma City Bus Station</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Dallas Bus Station</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>d6 Sat 08:35 FlixBus-us: Oklahoma City Bus Station -&gt; Dallas Bus Station</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>15</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>d6 Sat 11:30 FlixBus-us</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Dallas Bus Station</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Downtown Houston (Gray St.)</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>d6 Sat 11:50 DALLAS AREA RAPID TRANSIT: BACHMAN STATION -&gt; AKARD STATION</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>16</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>d6 Sat 16:48 Metropolitan Transit Authority of Harris County</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Theater District Rusk EB</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Magnolia Park Transit Center EB</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>d6 Sat 17:06 Metropolitan Transit Authority of Harris County: Theater District Rusk EB -&gt; Magnolia Park Transit Center EB</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>17</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>d6 Sat 18:35 Greyhound-us</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Houston Bus Station (Greyhound)</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Tallahassee (CK Steele Bus Plaza)</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>d6 Sat 22:00 Greyhound-us: Houston Bus Station (Greyhound) -&gt; Mobile Bus Station</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>18</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>d7 Sun 11:25 Greyhound-us</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Tallahassee (CK Steele Bus Plaza)</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Jacksonville (Downtown)</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>d7 Sun 17:10 Greyhound-us: Tallahassee (CK Steele Bus Plaza) -&gt; Jacksonville (Downtown)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>19</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>d7 Sun 15:00 Jacksonville Transportation Authority</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>JRTC Bay H</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Amtrak Station</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>d7 Sun 16:11 Amtrak: Jacksonville -&gt; Washington Union Station</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>20</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>d7 Sun 16:11 Amtrak</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Jacksonville</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Washington Union Station</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>wait 1 day(s) and catch the same bus, then continue</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>21</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>d8 Mon 06:50 Amtrak</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Washington Union Station</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Boston</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>wait 1 day(s) and catch the same bus, then continue</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>22</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>d8 Mon 14:15 Concord Coach Lines</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Boston South Station</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Portland, ME</t>
+        </is>
+      </c>
+      <c r="E24" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>d8 Mon 15:15 Concord Coach Lines: Boston South Station -&gt; Portland, ME</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>23</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>d8 Mon 16:45 Concord Coach Lines</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Portland, ME</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Boston South Station</t>
+        </is>
+      </c>
+      <c r="E25" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>d8 Mon 18:00 Concord Coach Lines: Portland, ME -&gt; Boston South Station</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>24</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>d8 Mon 19:30 Dartmouth Coach</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Boston South Station</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Hanover (Hanover Inn)</t>
+        </is>
+      </c>
+      <c r="E26" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>d8 Mon 21:30 Dartmouth Coach: Boston South Station -&gt; Hanover (Hanover Inn)</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>25</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>d9 Tue 03:00 Dartmouth Coach</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Hanover (Hanover Inn)</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Boston South Station</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>d9 Tue 04:35 Greyhound-us: White River Junction Bus Station -&gt; Boston (South Station)</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>26</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>d9 Tue 07:00 Amtrak</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Boston</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Washington Union Station</t>
+        </is>
+      </c>
+      <c r="E28" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>d9 Tue 07:15 FlixBus-us: Boston (South Station) -&gt; New York Midtown (31st St &amp; 8th Ave)</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>27</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>d9 Tue 15:57 Amtrak</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Washington Union Station</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Toledo</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>d9 Tue 17:50 Greyhound-us: Washington Union Station -&gt; Pittsburgh Intermodal Station</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>28</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>d10 Wed 06:30 Amtrak Chartered Vehicle</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Toledo</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Detroit</t>
+        </is>
+      </c>
+      <c r="E30" s="4" t="n">
+        <v>8.1</v>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>d10 Wed 07:55 Greyhound-us: Toledo Bus Stop -&gt; Detroit Bus Station</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>29</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>d10 Wed 07:44 Detroit Department of Transportation</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Woodward &amp; Baltimore</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Woodward &amp; State Fair</t>
+        </is>
+      </c>
+      <c r="E31" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>d10 Wed 09:35 Amtrak: Detroit -&gt; Chicago Union Station</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>30</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>d10 Wed 09:12 Amtrak</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Royal Oak Amtrak</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Chicago Union Station</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="n">
+        <v>21.4</v>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>d10 Wed 10:12 Detroit Department of Transportation: Jason Hargrove Transit Center - Bay 4 -&gt; Rosa Parks Transit Center - Bay 15</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>31</v>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>d10 Wed 14:10 Van Galder (Coach USA)</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>W Jackson Blvd, after S Clinton St (across from Union Station)</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Multi-Modal/Rental Car Facility</t>
+        </is>
+      </c>
+      <c r="E33" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>d10 Wed 15:05 Amtrak: Chicago Union Station -&gt; Milwaukee</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>32</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>d10 Wed 15:30 Wisconsin Coach Lines</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Multi-Modal/Rental Car Facility</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Kenosha Brat Stop</t>
+        </is>
+      </c>
+      <c r="E34" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>d10 Wed 16:30 Wisconsin Coach Lines: Multi-Modal/Rental Car Facility -&gt; Kenosha Brat Stop</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>33</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>d10 Wed 16:45 Wisconsin Coach Lines</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Kenosha Brat Stop</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>O'Hare International Airport - Terminal 2 Departures</t>
+        </is>
+      </c>
+      <c r="E35" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>d10 Wed 17:45 Wisconsin Coach Lines: Kenosha Brat Stop -&gt; O'Hare International Airport - Terminal 1 Departures</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>34</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>d10 Wed 17:37 Chicago Transit Authority</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>O'Hare</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Clinton-Blue</t>
+        </is>
+      </c>
+      <c r="E36" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>d10 Wed 17:45 Chicago Transit Authority: O'Hare -&gt; Clinton-Blue</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>35</v>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>d10 Wed 20:05 Amtrak</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Chicago Union Station</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Memphis</t>
+        </is>
+      </c>
+      <c r="E37" s="4" t="n">
+        <v>8.1</v>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>d10 Wed 22:50 Greyhound-us: Chicago Bus Station -&gt; Nashville Bus Station</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>36</v>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>d11 Thu 06:55 On foot (Big River Crossing, open 06:00-22:00)</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Memphis</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Arkansas line on Big River Crossing (on foot from Memphis Amtrak)</t>
+        </is>
+      </c>
+      <c r="E38" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>d11 Thu 07:05 On foot (Big River Crossing, open 06:00-22:00): Memphis -&gt; Arkansas line on Big River Crossing (on foot from Memphis Amtrak)</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>37</v>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>d11 Thu 07:40 On foot (Big River Crossing, open 06:00-22:00)</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Arkansas line on Big River Crossing (on foot from Memphis Amtrak)</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Memphis</t>
+        </is>
+      </c>
+      <c r="E39" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>d11 Thu 07:50 On foot (Big River Crossing, open 06:00-22:00): Arkansas line on Big River Crossing (on foot from Memphis Amtrak) -&gt; Memphis</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>38</v>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>d11 Thu 08:43 MATA</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>UNION AVENUE at 3RD STREET</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>WILLIAM HUDSON TRANSIT CENTER</t>
+        </is>
+      </c>
+      <c r="E40" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>d11 Thu 08:57 MATA: 3RD STREET at UNION AVENUE -&gt; WILLIAM HUDSON TRANSIT CENTER</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>39</v>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>d11 Thu 09:15 MATA</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>WILLIAM HUDSON TRANSIT CENTER</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>IRS</t>
+        </is>
+      </c>
+      <c r="E41" s="3" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>d11 Thu 09:45 MATA: WILLIAM HUDSON TRANSIT CENTER -&gt; JEFFERSON AVENUE at MONTGOMERY STREET</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:F39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -2793,7 +3947,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
redundancy: visited pins dropped, all targets on next-day replay, full-order target; clean results
Leaf script, nothing imports it.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/redundancy.xlsx
+++ b/docs/redundancy.xlsx
@@ -787,12 +787,12 @@
           <t>Oklahoma City</t>
         </is>
       </c>
-      <c r="E13" s="3" t="n">
-        <v>0</v>
+      <c r="E13" s="2" t="n">
+        <v>24</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>d13 Mon 04:00 Beeline Express: Newton -&gt; Oklahoma City</t>
+          <t>wait 1 day(s) and catch the same bus, then continue</t>
         </is>
       </c>
     </row>
@@ -1096,11 +1096,11 @@
         </is>
       </c>
       <c r="E24" s="2" t="n">
-        <v>57.4</v>
+        <v>24</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>d15 Wed 22:25 FlixBus-us: White River Junction Bus Station -&gt; Boston (South Station)</t>
+          <t>wait 1 day(s) and catch the same bus, then continue</t>
         </is>
       </c>
     </row>
@@ -1123,8 +1123,8 @@
           <t>Portland, ME</t>
         </is>
       </c>
-      <c r="E25" s="2" t="n">
-        <v>57.4</v>
+      <c r="E25" s="3" t="n">
+        <v>0</v>
       </c>
       <c r="F25" t="inlineStr">
         <is>
@@ -1151,8 +1151,8 @@
           <t>Boston South Station</t>
         </is>
       </c>
-      <c r="E26" s="2" t="n">
-        <v>57.4</v>
+      <c r="E26" s="3" t="n">
+        <v>0</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>
@@ -1179,12 +1179,12 @@
           <t>Ny Moynihan Train Hall At Penn Station</t>
         </is>
       </c>
-      <c r="E27" s="2" t="n">
-        <v>57.4</v>
+      <c r="E27" s="3" t="n">
+        <v>0</v>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>d16 Thu 07:00 Amtrak: Boston -&gt; Ny Moynihan Train Hall At Penn Station</t>
+          <t>d16 Thu 07:00 Amtrak: Boston -&gt; Newark</t>
         </is>
       </c>
     </row>
@@ -1207,12 +1207,12 @@
           <t>Harrisburg Bus Station</t>
         </is>
       </c>
-      <c r="E28" s="2" t="n">
-        <v>24</v>
+      <c r="E28" s="3" t="n">
+        <v>0</v>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>d16 Thu 11:33 Amtrak: Ny Moynihan Train Hall At Penn Station -&gt; White River Junction Amtrak Station</t>
+          <t>d16 Thu 11:06 Amtrak: Ny Moynihan Train Hall At Penn Station -&gt; Newark</t>
         </is>
       </c>
     </row>
@@ -1236,11 +1236,11 @@
         </is>
       </c>
       <c r="E29" s="2" t="n">
-        <v>57.4</v>
+        <v>24</v>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>d16 Thu 19:50 Greyhound-us: Harrisburg Bus Station -&gt; Indianapolis Bus Station</t>
+          <t>wait 1 day(s) and catch the same bus, then continue</t>
         </is>
       </c>
     </row>
@@ -1291,8 +1291,8 @@
           <t>Memphis Hilton, Ridge Lake Blvd (Vonlane)</t>
         </is>
       </c>
-      <c r="E31" s="2" t="n">
-        <v>24</v>
+      <c r="E31" s="3" t="n">
+        <v>0</v>
       </c>
       <c r="F31" t="inlineStr">
         <is>
@@ -1403,8 +1403,8 @@
           <t>Chicago Bus Station</t>
         </is>
       </c>
-      <c r="E35" s="2" t="n">
-        <v>24</v>
+      <c r="E35" s="3" t="n">
+        <v>0</v>
       </c>
       <c r="F35" t="inlineStr">
         <is>
@@ -1436,7 +1436,7 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>d18 Sat 06:05 Chicago Transit Authority: Clinton-Blue -&gt; Rosemont</t>
+          <t>d18 Sat 06:32 Metra: Chicago OTC -&gt; Kenosha</t>
         </is>
       </c>
     </row>
@@ -1684,7 +1684,7 @@
         </is>
       </c>
       <c r="E45" s="4" t="n">
-        <v>9.4</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="F45" t="inlineStr">
         <is>
@@ -2081,11 +2081,11 @@
         </is>
       </c>
       <c r="E14" s="2" t="n">
-        <v>144</v>
+        <v>24</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>d4 Thu 18:55 Greyhound-us: San Bernardino Depot -&gt; Las Vegas Bus Terminal</t>
+          <t>wait 1 day(s) and catch the same bus, then continue</t>
         </is>
       </c>
     </row>
@@ -2108,12 +2108,12 @@
           <t>Oklahoma City</t>
         </is>
       </c>
-      <c r="E15" s="3" t="n">
-        <v>0</v>
+      <c r="E15" s="2" t="n">
+        <v>24</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>d6 Sat 04:00 Beeline Express: Newton -&gt; Oklahoma City</t>
+          <t>d6 Sat 05:30 BeeLine Express-Village Travel: Newton (Amtrak) -&gt; Wichita</t>
         </is>
       </c>
     </row>
@@ -3597,12 +3597,12 @@
           <t>Oklahoma City</t>
         </is>
       </c>
-      <c r="E27" s="3" t="n">
-        <v>0</v>
+      <c r="E27" s="2" t="n">
+        <v>24</v>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>d16 Thu 04:00 Beeline Express: Newton -&gt; Oklahoma City</t>
+          <t>d16 Thu 05:30 BeeLine Express-Village Travel: Newton (Amtrak) -&gt; Wichita</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
redundancy: X's Sheridan miss 0 h (start next day, Fri 22:20 gives 231.7 h), Billings miss +24 h
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/redundancy.xlsx
+++ b/docs/redundancy.xlsx
@@ -507,12 +507,12 @@
           <t>Billings</t>
         </is>
       </c>
-      <c r="E3" s="2" t="n">
-        <v>144</v>
+      <c r="E3" s="3" t="n">
+        <v>0</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>d10 Fri 06:35 Jefferson Lines: Sheridan WY Taco Bell 1655 Coffeen Ave (Jefferson) -&gt; Vivian</t>
+          <t>first bus: start the next day instead; the clock starts at the first bus. Fri Nov 13 22:20 start gives 231.7 h (out/omni/x_fri.log)</t>
         </is>
       </c>
     </row>
@@ -536,11 +536,11 @@
         </is>
       </c>
       <c r="E4" s="2" t="n">
-        <v>144</v>
+        <v>24</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>d10 Fri 11:30 Jefferson Lines: Billings -&gt; Whitefish</t>
+          <t>Billings -&gt; Spokane is daily: next day's bus, same route, +24 h (Fri start runs the same shape, out/omni/x_fri.log)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
redundancy: real record (KC-Tulsa-Dallas-El Paso-LA, 238.83 h) as Record; search's Omnibus variant as Record-Omnibus
Leaf script, nothing imports it; regress skipped.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/redundancy.xlsx
+++ b/docs/redundancy.xlsx
@@ -11,6 +11,7 @@
     <sheet name="Moorhead" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Control" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Record" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Record-Omnibus" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -3953,6 +3954,935 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:F33"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="4" customWidth="1" min="1" max="1"/>
+    <col width="36" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="100" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Record: 238.83 h from the first bus. Miss each ride by one minute and replay the rest.</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>missed</t>
+        </is>
+      </c>
+      <c r="C2" s="1" t="inlineStr">
+        <is>
+          <t>from</t>
+        </is>
+      </c>
+      <c r="D2" s="1" t="inlineStr">
+        <is>
+          <t>to</t>
+        </is>
+      </c>
+      <c r="E2" s="1" t="inlineStr">
+        <is>
+          <t>cost h</t>
+        </is>
+      </c>
+      <c r="F2" s="1" t="inlineStr">
+        <is>
+          <t>recovery starts with</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>d1 Thu 04:35 Greyhound-us</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>White River Junction Bus Station</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Boston (South Station)</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>d1 Thu 06:40 Dartmouth Coach: Hanover (Hanover Inn) -&gt; Boston South Station</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>2</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>d1 Thu 08:00 Concord Coach Lines</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Boston South Station</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Portland, ME</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>d1 Thu 08:50 Amtrak: Boston -&gt; Portland</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>3</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>d1 Thu 10:30 Concord Coach Lines</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Portland, ME</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Boston South Station</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>d1 Thu 11:30 Concord Coach Lines: Portland, ME -&gt; Boston South Station</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>4</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>d1 Thu 13:00 Amtrak</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Boston</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Washington Union Station</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>wait 1 day(s) and catch the same bus, then continue</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>5</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>d1 Thu 21:45 FlixBus-us</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Washington Union Station</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Jacksonville (Downtown)</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>d1 Thu 22:45 FlixBus-us: Washington Union Station -&gt; Charlotte Bus Station</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>6</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>d2 Fri 16:15 Greyhound-us</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Jacksonville (Downtown)</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Tallahassee (CK Steele Bus Plaza)</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>d2 Fri 16:30 FlixBus-us: Jacksonville (Downtown) -&gt; Atlanta Bus Station</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>7</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>d2 Fri 20:50 Greyhound-us</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Tallahassee (CK Steele Bus Plaza)</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Baton Rouge Bus Station</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>wait 1 day(s) and catch the same bus, then continue</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>8</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>d3 Sat 06:05 Greyhound-us</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Baton Rouge Bus Station</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>St Louis Bus Station</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>wait 1 day(s) and catch the same bus, then continue</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>9</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>d3 Sat 23:45 Greyhound-us</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>St Louis Bus Station</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Kansas City Bus Station</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>d4 Sun 01:20 Greyhound-us: St Louis Bus Station -&gt; Oklahoma City Bus Station</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>10</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>d4 Sun 05:20 Jefferson Lines</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Kansas City Bus Station</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Tulsa</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>d4 Sun 06:15 Greyhound-us: Kansas City Bus Station -&gt; Oklahoma City Bus Station</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>11</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>d4 Sun 10:50 Greyhound-us</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Tulsa Bus Station</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Dallas Bus Station</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>d4 Sun 16:45 Greyhound-us: Tulsa Bus Station -&gt; Amarillo Multimodal Transfer Sta</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>12</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>d4 Sun 19:00 Greyhound-us</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Dallas Bus Station</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>El Paso Bus Station (W San Antonio St)</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>d4 Sun 23:50 Greyhound-us: Dallas Bus Station -&gt; Los Angeles Union Station</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>13</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>d5 Mon 07:00 Greyhound-us</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>El Paso Bus Station (W San Antonio St)</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Los Angeles Union Station</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>d5 Mon 12:35 Greyhound-us: El Paso Bus Station (W San Antonio St) -&gt; Los Angeles Union Station</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>14</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>d6 Tue 00:30 Greyhound-us</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Los Angeles Union Station</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Las Vegas Bus Terminal</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>d6 Tue 06:25 Greyhound-us: Los Angeles Union Station -&gt; Las Vegas Bus Terminal</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>15</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>d6 Tue 09:00 Salt Lake Express</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Las Vegas (Airport)</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Saint George (Shop)</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>d6 Tue 11:00 Salt Lake Express: Las Vegas (Airport) -&gt; Saint George (Shop)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>16</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>d6 Tue 16:05 Salt Lake Express</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Saint George (Shop)</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Salt Lake City (Airport)</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>d7 Wed 03:35 Salt Lake Express: Saint George (Shop) -&gt; Salt Lake City (Airport)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>17</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>d6 Tue 22:30 Salt Lake Express</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Salt Lake City (Airport)</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Pocatello (Transit Depot)</t>
+        </is>
+      </c>
+      <c r="E19" s="4" t="n">
+        <v>18.5</v>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>d6 Tue 22:39 Utah Transit Authority: Airport Station -&gt; North Temple Bridge/Guadalupe</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>18</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>d7 Wed 03:40 Salt Lake Express</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Pocatello (Transit Depot)</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Boise (Airport)</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>d7 Wed 13:25 Salt Lake Express: Pocatello (Transit Depot) -&gt; Boise (Airport)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>19</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>d7 Wed 08:15 Northwestern Stage Lines</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Boise (Airport)</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Pasco Bus Stop</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>d7 Wed 10:30 Greyhound-us: Boise (Chevron) -&gt; Pasco Bus Stop</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>20</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>d7 Wed 14:40 FlixBus-us</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Pasco Bus Stop</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Spokane Station</t>
+        </is>
+      </c>
+      <c r="E22" s="4" t="n">
+        <v>18.5</v>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>d7 Wed 15:00 Northwestern Stage Lines: Pasco Bus Stop -&gt; Spokane</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>21</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>d7 Wed 17:10 Jefferson Lines</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Spokane</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Billings</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>d8 Thu 17:10 Jefferson Lines: Spokane -&gt; Billings</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>22</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>d8 Thu 04:30 Jefferson Lines</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Billings</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Buffalo</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>d9 Fri 04:30 Jefferson Lines: Billings -&gt; Buffalo</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>23</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>d8 Thu 07:20 Express Arrow</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Buffalo</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Denver</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>d9 Fri 07:20 Express Arrow: Buffalo -&gt; Denver</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>24</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>d8 Thu 18:59 Amtrak</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Denver</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Omaha Amtrak Station</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>d9 Fri 09:25 Express Arrow: Denver -&gt; Omaha</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>25</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>d9 Fri 06:15 Jefferson Lines</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Omaha</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Sioux Falls</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>d10 Sat 06:15 Jefferson Lines: Omaha -&gt; Sioux Falls</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>26</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>d9 Fri 10:00 Jefferson Lines</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Sioux Falls</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Fargo</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>d9 Fri 10:30 Jefferson Lines: Sioux Falls -&gt; Minneapolis</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>27</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>d9 Fri 16:40 Jefferson Lines</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Fargo</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Minneapolis</t>
+        </is>
+      </c>
+      <c r="E29" s="4" t="n">
+        <v>18.5</v>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>d9 Fri 17:45 MATBUS: MATBUS - 222 4th St. N -&gt; Shelter 139 (US Bank)</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>28</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>d10 Sat 00:15 Greyhound-us</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Minneapolis Bus Station</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Chicago Bus Station</t>
+        </is>
+      </c>
+      <c r="E30" s="4" t="n">
+        <v>18.5</v>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>d10 Sat 07:45 FlixBus-us: Minneapolis Bus Station -&gt; Madison (Madison Campus WI)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>29</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>d10 Sat 09:05 Barons Bus Lines</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Chicago</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Toledo (Amtrak)</t>
+        </is>
+      </c>
+      <c r="E31" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>d10 Sat 09:13 Chicago Transit Authority: Jefferson &amp; Harrison -&gt; Randolph &amp; Michigan</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>30</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>d10 Sat 15:35 Greyhound-us</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Toledo Bus Stop</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Detroit Bus Station</t>
+        </is>
+      </c>
+      <c r="E32" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>d10 Sat 16:55 Greyhound-us: Toledo Bus Stop -&gt; Detroit Bus Station</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>31</v>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>d10 Sat 19:55 Greyhound-us</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Detroit Bus Station</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Huntington Bus Stop</t>
+        </is>
+      </c>
+      <c r="E33" s="4" t="n">
+        <v>16.4</v>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>d10 Sat 21:30 Amtrak Chartered Vehicle: Detroit -&gt; Toledo</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:F32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -3967,7 +4897,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Record: 239.00 h. Miss each ride by one minute and replay the rest.</t>
+          <t>Record-Omnibus: 238.83 h from the first bus (search variant of the record: Omnibus KC 13:01 -&gt; Tucumcari). Miss each ride by one minute and replay the rest.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Overnight Oct 16-17: focused searches hold (X 232.1, Moorhead 235.8, control 237.5, record 238.8), sweep 8 best 244.4; redundancy refreshed
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/redundancy.xlsx
+++ b/docs/redundancy.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F45"/>
+  <dimension ref="A1:F48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -453,7 +453,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>X: 231.85 h. Miss each ride by one minute and replay the rest.</t>
+          <t>X: 232.13 h from the first bus. Miss each ride by one minute and replay the rest.</t>
         </is>
       </c>
     </row>
@@ -508,12 +508,12 @@
           <t>Billings</t>
         </is>
       </c>
-      <c r="E3" s="3" t="n">
-        <v>0</v>
+      <c r="E3" s="2" t="n">
+        <v>120</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>first bus: start the next day instead; the clock starts at the first bus. Fri Nov 13 22:20 start gives 231.7 h (out/omni/x_fri.log)</t>
+          <t>d10 Fri 06:35 Jefferson Lines: Sheridan WY Taco Bell 1655 Coffeen Ave (Jefferson) -&gt; Vivian</t>
         </is>
       </c>
     </row>
@@ -537,11 +537,11 @@
         </is>
       </c>
       <c r="E4" s="2" t="n">
-        <v>24</v>
+        <v>120</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Billings -&gt; Spokane is daily: next day's bus, same route, +24 h (Fri start runs the same shape, out/omni/x_fri.log)</t>
+          <t>d11 Sat 01:30 Jefferson Lines: Billings -&gt; Spokane</t>
         </is>
       </c>
     </row>
@@ -607,17 +607,17 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>d11 Sat 04:45 Salt Lake Express</t>
+          <t>d11 Sat 04:08 Utah Transit Authority</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Salt Lake City (Airport)</t>
+          <t>North Temple Station (Bay A)</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Saint George (Bluff St Office)</t>
+          <t>State St / Harvard Ave (SB)</t>
         </is>
       </c>
       <c r="E7" s="3" t="n">
@@ -625,7 +625,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>d11 Sat 06:00 Salt Lake Express: Salt Lake City (Airport) -&gt; Saint George (Bluff St Office)</t>
+          <t>d11 Sat 04:28 Utah Transit Authority: North Temple / 600 W (EB) -&gt; 200 S / Main St (EB)</t>
         </is>
       </c>
     </row>
@@ -635,17 +635,17 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>d11 Sat 10:30 Salt Lake Express</t>
+          <t>d11 Sat 04:46 Utah Transit Authority</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Saint George (Bluff St Office)</t>
+          <t>Ballpark Station</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Las Vegas (Airport)</t>
+          <t>Airport Station</t>
         </is>
       </c>
       <c r="E8" s="3" t="n">
@@ -653,7 +653,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>d11 Sat 12:15 Salt Lake Express: Saint George (Shop) -&gt; Las Vegas (Airport)</t>
+          <t>d11 Sat 05:01 Utah Transit Authority: Ballpark Station -&gt; Airport Station</t>
         </is>
       </c>
     </row>
@@ -663,17 +663,17 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t xml:space="preserve">d11 Sat 11:57 Regional Transportation Commission of Southern Nevada </t>
+          <t>d11 Sat 06:00 St George Shuttle</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Harry Reid Intl Airport Zero Level</t>
+          <t>Salt Lake City (Airport)</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>South Strip Transit Terminal Bay 6</t>
+          <t>Las Vegas (Airport)</t>
         </is>
       </c>
       <c r="E9" s="3" t="n">
@@ -681,7 +681,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>d11 Sat 12:09 Regional Transportation Commission of Southern Nevada : Harry Reid Intl Airport Zero Level -&gt; South Strip Transit Terminal Bay 6</t>
+          <t>d11 Sat 06:45 Salt Lake Express: Salt Lake City (Airport) -&gt; Saint George (Bluff St Office)</t>
         </is>
       </c>
     </row>
@@ -691,17 +691,17 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>d11 Sat 12:35 Alvand Transportation</t>
+          <t xml:space="preserve">d11 Sat 13:19 Regional Transportation Commission of Southern Nevada </t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Las Vegas Amtrak Bus Stop</t>
+          <t>Harry Reid Intl Airport Zero Level</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>San Bernardino</t>
+          <t>NB University Ctr before Flamingo</t>
         </is>
       </c>
       <c r="E10" s="3" t="n">
@@ -709,7 +709,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>d11 Sat 14:00 Greyhound-us: Las Vegas Bus Terminal -&gt; San Bernardino Depot</t>
+          <t>d11 Sat 13:28 Regional Transportation Commission of Southern Nevada : Harry Reid Intl Airport Zero Level -&gt; NB Maryland after Flamingo</t>
         </is>
       </c>
     </row>
@@ -719,17 +719,17 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>d11 Sat 17:38 Omnitrans</t>
+          <t xml:space="preserve">d11 Sat 13:50 Regional Transportation Commission of Southern Nevada </t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>San Bernardino Transit Center</t>
+          <t>EB Flamingo after Hospitality</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Vine Street Mobility Hub</t>
+          <t>EB Flamingo after Eastern</t>
         </is>
       </c>
       <c r="E11" s="3" t="n">
@@ -737,7 +737,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>d11 Sat 17:50 Omnitrans: San Bernardino Transit Center -&gt; 2nd Street @ L Street</t>
+          <t>d11 Sat 14:05 Regional Transportation Commission of Southern Nevada : EB Flamingo after Hospitality -&gt; EB Flamingo after Maryland</t>
         </is>
       </c>
     </row>
@@ -747,25 +747,25 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>d11 Sat 18:18 Amtrak</t>
+          <t xml:space="preserve">d11 Sat 14:13 Regional Transportation Commission of Southern Nevada </t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Riverside</t>
+          <t>NB Eastern after Flamingo</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Newton</t>
-        </is>
-      </c>
-      <c r="E12" s="2" t="n">
-        <v>24</v>
+          <t>NB Civic Center after Owens</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="n">
+        <v>0</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>wait 1 day(s) and catch the same bus, then continue</t>
+          <t>d11 Sat 14:21 Regional Transportation Commission of Southern Nevada : WB Flamingo after Eastern -&gt; WB Flamingo after Algonquin</t>
         </is>
       </c>
     </row>
@@ -775,25 +775,25 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>d13 Mon 03:00 BeeLine Express-Village Travel</t>
+          <t>d11 Sat 15:00 702 Shuttles</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Newton (Amtrak)</t>
+          <t>Las Vegas 1404 N Eastern Ave (702 Shuttles)</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Oklahoma City</t>
+          <t>Barstow East Main St 1611 (702 Shuttles)</t>
         </is>
       </c>
       <c r="E13" s="2" t="n">
-        <v>24</v>
+        <v>120</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>wait 1 day(s) and catch the same bus, then continue</t>
+          <t>d11 Sat 18:00 702 Shuttles: Las Vegas 1404 N Eastern Ave (702 Shuttles) -&gt; El Monte Valley Blvd (702 Shuttles)</t>
         </is>
       </c>
     </row>
@@ -803,25 +803,25 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>d13 Mon 06:55 Greyhound-us</t>
+          <t>d11 Sat 20:47 Amtrak</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Oklahoma City Bus Station</t>
+          <t>Barstow</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Dallas Bus Station</t>
-        </is>
-      </c>
-      <c r="E14" s="3" t="n">
-        <v>0</v>
+          <t>Newton</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="n">
+        <v>120</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>d13 Mon 08:35 FlixBus-us: Oklahoma City Bus Station -&gt; Dallas Bus Station</t>
+          <t>d11 Sat 22:25 FlixBus-us: Barstow Station -&gt; Las Vegas Strip (Las Vegas Blvd)</t>
         </is>
       </c>
     </row>
@@ -831,25 +831,25 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>d13 Mon 11:30 FlixBus-us</t>
+          <t>d13 Mon 03:00 BeeLine Express-Village Travel</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Dallas Bus Station</t>
+          <t>Newton (Amtrak)</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Downtown Houston (Gray St.)</t>
-        </is>
-      </c>
-      <c r="E15" s="3" t="n">
-        <v>0</v>
+          <t>Oklahoma City</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="n">
+        <v>96</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>d13 Mon 11:50 DALLAS AREA RAPID TRANSIT: BACHMAN STATION -&gt; AKARD STATION</t>
+          <t>d13 Mon 05:30 BeeLine Express-Village Travel: Newton (Amtrak) -&gt; Wichita</t>
         </is>
       </c>
     </row>
@@ -859,17 +859,17 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>d13 Mon 16:50 Metropolitan Transit Authority of Harris County</t>
+          <t>d13 Mon 06:55 Greyhound-us</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Central Station Rusk EB</t>
+          <t>Oklahoma City Bus Station</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Magnolia Park Transit Center EB</t>
+          <t>Dallas Bus Station</t>
         </is>
       </c>
       <c r="E16" s="3" t="n">
@@ -877,7 +877,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>d13 Mon 17:02 Metropolitan Transit Authority of Harris County: Central Station Rusk EB -&gt; Magnolia Park Transit Center EB</t>
+          <t>d13 Mon 08:35 FlixBus-us: Oklahoma City Bus Station -&gt; Dallas Bus Station</t>
         </is>
       </c>
     </row>
@@ -887,25 +887,25 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>d13 Mon 18:35 Greyhound-us</t>
+          <t>d13 Mon 11:30 FlixBus-us</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Houston Bus Station (Greyhound)</t>
+          <t>Dallas Bus Station</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Tallahassee (CK Steele Bus Plaza)</t>
-        </is>
-      </c>
-      <c r="E17" s="2" t="n">
-        <v>24</v>
+          <t>Downtown Houston (Gray St.)</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="n">
+        <v>0</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>wait 1 day(s) and catch the same bus, then continue</t>
+          <t>d13 Mon 11:50 DALLAS AREA RAPID TRANSIT: BACHMAN STATION -&gt; AKARD STATION</t>
         </is>
       </c>
     </row>
@@ -915,25 +915,25 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>d14 Tue 11:25 Greyhound-us</t>
+          <t>d13 Mon 16:50 Metropolitan Transit Authority of Harris County</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Tallahassee (CK Steele Bus Plaza)</t>
+          <t>Central Station Rusk EB</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Jacksonville (Downtown)</t>
-        </is>
-      </c>
-      <c r="E18" s="2" t="n">
-        <v>24</v>
+          <t>Magnolia Park Transit Center EB</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="n">
+        <v>0</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>wait 1 day(s) and catch the same bus, then continue</t>
+          <t>d13 Mon 17:02 Metropolitan Transit Authority of Harris County: Central Station Rusk EB -&gt; Magnolia Park Transit Center EB</t>
         </is>
       </c>
     </row>
@@ -943,25 +943,25 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>d14 Tue 15:00 Jacksonville Transportation Authority</t>
+          <t>d13 Mon 18:35 Greyhound-us</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>JRTC Bay H</t>
+          <t>Houston Bus Station (Greyhound)</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Amtrak Station</t>
-        </is>
-      </c>
-      <c r="E19" s="3" t="n">
-        <v>0</v>
+          <t>Tallahassee (CK Steele Bus Plaza)</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="n">
+        <v>96</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>d14 Tue 16:11 Amtrak: Jacksonville -&gt; Washington Union Station</t>
+          <t>d13 Mon 22:00 Greyhound-us: Houston Bus Station (Greyhound) -&gt; Mobile Bus Station</t>
         </is>
       </c>
     </row>
@@ -971,25 +971,25 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>d14 Tue 16:11 Amtrak</t>
+          <t>d14 Tue 11:25 Greyhound-us</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Jacksonville</t>
+          <t>Tallahassee (CK Steele Bus Plaza)</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Washington Union Station</t>
+          <t>Jacksonville (Downtown)</t>
         </is>
       </c>
       <c r="E20" s="2" t="n">
-        <v>24</v>
+        <v>79.8</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>d14 Tue 16:27 Jacksonville Transportation Authority: Amtrak Station -&gt; JRTC Bay H</t>
+          <t>d14 Tue 12:50 Greyhound-us: Tallahassee (CK Steele Bus Plaza) -&gt; Atlanta Bus Station</t>
         </is>
       </c>
     </row>
@@ -999,17 +999,17 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>d15 Wed 06:50 Amtrak</t>
+          <t>d14 Tue 15:00 Jacksonville Transportation Authority</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Washington Union Station</t>
+          <t>JRTC Bay H</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Boston</t>
+          <t>Amtrak Station</t>
         </is>
       </c>
       <c r="E21" s="2" t="n">
@@ -1017,7 +1017,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>wait 1 day(s) and catch the same bus, then continue</t>
+          <t>d14 Tue 15:30 Jacksonville Transportation Authority: JRTC Bay H -&gt; Amtrak Station</t>
         </is>
       </c>
     </row>
@@ -1027,17 +1027,17 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>d15 Wed 14:30 Dartmouth Coach</t>
+          <t>d14 Tue 16:11 Amtrak</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Boston South Station</t>
+          <t>Jacksonville</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Hanover (Hanover Inn)</t>
+          <t>Washington Union Station</t>
         </is>
       </c>
       <c r="E22" s="2" t="n">
@@ -1045,7 +1045,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>wait 1 day(s) and catch the same bus, then continue</t>
+          <t>d14 Tue 16:27 Jacksonville Transportation Authority: Amtrak Station -&gt; JRTC Bay H</t>
         </is>
       </c>
     </row>
@@ -1055,25 +1055,25 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>d15 Wed 17:10 Advance Transit</t>
+          <t>d15 Wed 06:50 Amtrak</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Main at Allen</t>
+          <t>Washington Union Station</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Sykes Ave @ Greyhound</t>
+          <t>Boston</t>
         </is>
       </c>
       <c r="E23" s="2" t="n">
-        <v>24</v>
+        <v>55.8</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>wait 1 day(s) and catch the same bus, then continue</t>
+          <t>d15 Wed 07:10 Amtrak: Washington Union Station -&gt; Stamford Amtrak Station</t>
         </is>
       </c>
     </row>
@@ -1083,17 +1083,17 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>d15 Wed 17:55 Greyhound-us</t>
+          <t>d15 Wed 14:30 Dartmouth Coach</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>White River Junction Bus Station</t>
+          <t>Boston South Station</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Boston (South Station)</t>
+          <t>Hanover (Hanover Inn)</t>
         </is>
       </c>
       <c r="E24" s="2" t="n">
@@ -1101,7 +1101,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>wait 1 day(s) and catch the same bus, then continue</t>
+          <t>d15 Wed 15:30 Dartmouth Coach: Boston South Station -&gt; Hanover (Hanover Inn)</t>
         </is>
       </c>
     </row>
@@ -1111,25 +1111,25 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>d15 Wed 20:25 Concord Coach Lines</t>
+          <t>d15 Wed 17:10 Advance Transit</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Boston South Station</t>
+          <t>Main at Allen</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Portland, ME</t>
-        </is>
-      </c>
-      <c r="E25" s="3" t="n">
-        <v>0</v>
+          <t>Sykes Ave @ Greyhound</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="n">
+        <v>24</v>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>d15 Wed 20:40 Plymouth &amp; Brockton Street Railway Co.: South Station Transp. Ctr -&gt; Logan International Airport</t>
+          <t>d15 Wed 17:23 Advance Transit: Hanover Inn -&gt; Vail DMS</t>
         </is>
       </c>
     </row>
@@ -1139,25 +1139,25 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>d16 Thu 03:15 Concord Coach Lines</t>
+          <t>d15 Wed 17:55 Greyhound-us</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Portland, ME</t>
+          <t>White River Junction Bus Station</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Boston South Station</t>
-        </is>
-      </c>
-      <c r="E26" s="3" t="n">
-        <v>0</v>
+          <t>Boston (South Station)</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="n">
+        <v>24</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>d16 Thu 04:15 Concord Coach Lines: Portland, ME -&gt; Boston South Station</t>
+          <t>d15 Wed 22:25 FlixBus-us: White River Junction Bus Station -&gt; Boston (South Station)</t>
         </is>
       </c>
     </row>
@@ -1167,17 +1167,17 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>d16 Thu 06:10 Amtrak</t>
+          <t>d15 Wed 20:25 Concord Coach Lines</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Boston</t>
+          <t>Boston South Station</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Ny Moynihan Train Hall At Penn Station</t>
+          <t>Portland, ME</t>
         </is>
       </c>
       <c r="E27" s="3" t="n">
@@ -1185,7 +1185,7 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>d16 Thu 07:00 Amtrak: Boston -&gt; Newark</t>
+          <t>d15 Wed 20:40 Plymouth &amp; Brockton Street Railway Co.: South Station Transp. Ctr -&gt; Logan International Airport</t>
         </is>
       </c>
     </row>
@@ -1195,17 +1195,17 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>d16 Thu 10:45 FlixBus-us</t>
+          <t>d16 Thu 03:15 Concord Coach Lines</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>New York Midtown (31st St &amp; 8th Ave)</t>
+          <t>Portland, ME</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Harrisburg Bus Station</t>
+          <t>Boston South Station</t>
         </is>
       </c>
       <c r="E28" s="3" t="n">
@@ -1213,7 +1213,7 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>d16 Thu 11:06 Amtrak: Ny Moynihan Train Hall At Penn Station -&gt; Newark</t>
+          <t>d16 Thu 04:15 Concord Coach Lines: Portland, ME -&gt; Boston South Station</t>
         </is>
       </c>
     </row>
@@ -1223,25 +1223,25 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>d16 Thu 14:50 Greyhound-us</t>
+          <t>d16 Thu 06:10 Amtrak</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Harrisburg Bus Station</t>
+          <t>Boston</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Indianapolis Bus Station</t>
-        </is>
-      </c>
-      <c r="E29" s="2" t="n">
-        <v>24</v>
+          <t>Ny Moynihan Train Hall At Penn Station</t>
+        </is>
+      </c>
+      <c r="E29" s="3" t="n">
+        <v>0</v>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>wait 1 day(s) and catch the same bus, then continue</t>
+          <t>d16 Thu 07:00 Amtrak: Boston -&gt; Newark</t>
         </is>
       </c>
     </row>
@@ -1251,25 +1251,25 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>d17 Fri 04:40 Greyhound-us</t>
+          <t>d16 Thu 10:45 FlixBus-us</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Indianapolis Bus Station</t>
+          <t>New York Midtown (31st St &amp; 8th Ave)</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Nashville Bus Station</t>
-        </is>
-      </c>
-      <c r="E30" s="2" t="n">
-        <v>24</v>
+          <t>Harrisburg Bus Station</t>
+        </is>
+      </c>
+      <c r="E30" s="3" t="n">
+        <v>0</v>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>d17 Fri 05:20 Greyhound-us: Indianapolis Bus Station -&gt; Lafayette Bus Stop</t>
+          <t>d16 Thu 11:06 Amtrak: Ny Moynihan Train Hall At Penn Station -&gt; Newark</t>
         </is>
       </c>
     </row>
@@ -1279,25 +1279,25 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>d17 Fri 10:00 Vonlane</t>
+          <t>d16 Thu 14:50 Greyhound-us</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Nashville Omni Downtown (Vonlane)</t>
+          <t>Harrisburg Bus Station</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Memphis Hilton, Ridge Lake Blvd (Vonlane)</t>
-        </is>
-      </c>
-      <c r="E31" s="3" t="n">
-        <v>0</v>
+          <t>Indianapolis Bus Station</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="n">
+        <v>24</v>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>d17 Fri 11:30 FlixBus-us: Nashville Bus Station -&gt; Memphis Bus Station</t>
+          <t>d16 Thu 19:50 Greyhound-us: Harrisburg Bus Station -&gt; Indianapolis Bus Station</t>
         </is>
       </c>
     </row>
@@ -1307,25 +1307,25 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>d17 Fri 14:15 MATA</t>
+          <t>d17 Fri 04:40 Greyhound-us</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>GETWELL ROAD at ALLENBROOKE COVE</t>
+          <t>Indianapolis Bus Station</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>IRS</t>
-        </is>
-      </c>
-      <c r="E32" s="3" t="n">
-        <v>0</v>
+          <t>Nashville Bus Station</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="n">
+        <v>24</v>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>d17 Fri 14:26 MATA: AMERICAN WAY TRANSIT CENTER -&gt; WINCHESTER ROAD at RIVERDALE ROAD</t>
+          <t>d17 Fri 05:20 Greyhound-us: Indianapolis Bus Station -&gt; Lafayette Bus Stop</t>
         </is>
       </c>
     </row>
@@ -1335,17 +1335,17 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>d17 Fri 15:39 MATA</t>
+          <t>d17 Fri 10:00 Vonlane</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>IRS</t>
+          <t>Nashville Omni Downtown (Vonlane)</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>AIRWAYS TRANSIT CENTER</t>
+          <t>Memphis Hilton, Ridge Lake Blvd (Vonlane)</t>
         </is>
       </c>
       <c r="E33" s="3" t="n">
@@ -1353,7 +1353,7 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>d17 Fri 16:15 MATA: IRS -&gt; AIRWAYS TRANSIT CENTER</t>
+          <t>d17 Fri 11:30 FlixBus-us: Nashville Bus Station -&gt; Memphis Bus Station</t>
         </is>
       </c>
     </row>
@@ -1363,25 +1363,25 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>d17 Fri 17:45 Greyhound-us</t>
+          <t>d17 Fri 13:56 MATA</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Memphis Bus Station</t>
+          <t>POPLAR AVENUE at SHADY GROVE ROAD</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>St Louis Bus Station</t>
-        </is>
-      </c>
-      <c r="E34" s="2" t="n">
-        <v>24</v>
+          <t>POPLAR AVENUE at CLEVELAND STREET</t>
+        </is>
+      </c>
+      <c r="E34" s="3" t="n">
+        <v>0</v>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>d17 Fri 18:12 MATA: AIRWAYS TRANSIT CENTER -&gt; GE PATTERSON AVENUE at MAIN STREET</t>
+          <t>d17 Fri 14:30 MATA: PRIMACY PARKWAY at RIDGEWAY ROAD -&gt; BELLEVUE BOULEVARD at MCLEMORE AVENUE</t>
         </is>
       </c>
     </row>
@@ -1391,17 +1391,17 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>d17 Fri 23:30 FlixBus-us</t>
+          <t>d17 Fri 14:54 MATA</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>St Louis Bus Station</t>
+          <t>CLEVELAND STREET at LARKIN AVENUE</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Chicago Bus Station</t>
+          <t>HOLMES at LOCH LOMOND</t>
         </is>
       </c>
       <c r="E35" s="3" t="n">
@@ -1409,7 +1409,7 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>d17 Fri 23:45 FlixBus-us: St Louis Bus Station -&gt; Carbondale Intermodal Station</t>
+          <t>d17 Fri 15:06 MATA: CLEVELAND STREET at LARKIN AVENUE -&gt; WATKINS STREET at HENRY AVENUE</t>
         </is>
       </c>
     </row>
@@ -1419,17 +1419,17 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>d18 Sat 05:50 Chicago Transit Authority</t>
+          <t>d17 Fri 16:24 MATA</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Clinton-Blue</t>
+          <t>HOLMES ROAD at MILLBRANCH ROAD</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Rosemont</t>
+          <t>ELVIS PRESLEY BOULEVARD at SHELBY DRIVE</t>
         </is>
       </c>
       <c r="E36" s="3" t="n">
@@ -1437,7 +1437,7 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>d18 Sat 06:32 Metra: Chicago OTC -&gt; Kenosha</t>
+          <t>d17 Fri 17:02 MATA: HOLMES at ELVIS PRESLEY -&gt; AIRWAYS TRANSIT CENTER</t>
         </is>
       </c>
     </row>
@@ -1447,17 +1447,17 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>d18 Sat 07:30 Wisconsin Coach Lines</t>
+          <t>d17 Fri 16:42 MATA</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Multi-Modal/Rental Car Facility</t>
+          <t>SHELBY DRIVE at ELVIS PRESLEY BOULEVARD</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Kenosha Brat Stop</t>
+          <t>WINCHESTER ROAD at BOEINGSHIRE DRIVE</t>
         </is>
       </c>
       <c r="E37" s="3" t="n">
@@ -1465,7 +1465,7 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>d18 Sat 09:30 Wisconsin Coach Lines: Multi-Modal/Rental Car Facility -&gt; Kenosha Brat Stop</t>
+          <t>d17 Fri 16:58 MATA: Elvis Presley-Haledale -&gt; AIRWAYS TRANSIT CENTER</t>
         </is>
       </c>
     </row>
@@ -1475,25 +1475,25 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>d18 Sat 08:45 Wisconsin Coach Lines</t>
+          <t>d17 Fri 17:45 Greyhound-us</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Kenosha Brat Stop</t>
+          <t>Memphis Bus Station</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>O'Hare International Airport - Terminal 2 Departures</t>
-        </is>
-      </c>
-      <c r="E38" s="3" t="n">
-        <v>0</v>
+          <t>St Louis Bus Station</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="n">
+        <v>24</v>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>d18 Sat 10:45 Wisconsin Coach Lines: Kenosha Brat Stop -&gt; O'Hare International Airport - Terminal 2 Departures</t>
+          <t>d17 Fri 18:12 MATA: AIRWAYS TRANSIT CENTER -&gt; GE PATTERSON AVENUE at MAIN STREET</t>
         </is>
       </c>
     </row>
@@ -1503,17 +1503,17 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>d18 Sat 09:42 Chicago Transit Authority</t>
+          <t>d17 Fri 23:30 FlixBus-us</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>O'Hare</t>
+          <t>St Louis Bus Station</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Clark/Lake (Subway)</t>
+          <t>Chicago Bus Station</t>
         </is>
       </c>
       <c r="E39" s="3" t="n">
@@ -1521,7 +1521,7 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>d18 Sat 09:51 Chicago Transit Authority: O'Hare -&gt; Clark/Lake (Subway)</t>
+          <t>d17 Fri 23:45 FlixBus-us: St Louis Bus Station -&gt; Carbondale Intermodal Station</t>
         </is>
       </c>
     </row>
@@ -1531,17 +1531,17 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>d18 Sat 10:29 Chicago Transit Authority</t>
+          <t>d18 Sat 06:32 Metra</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Clark/Lake (Elevated)</t>
+          <t>Chicago OTC</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>35-Bronzeville-IIT</t>
+          <t>Kenosha</t>
         </is>
       </c>
       <c r="E40" s="3" t="n">
@@ -1549,7 +1549,7 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>d18 Sat 10:39 Chicago Transit Authority: Clark/Lake (Elevated) -&gt; 35-Bronzeville-IIT</t>
+          <t>d18 Sat 07:15 Van Galder (Coach USA): W Jackson Blvd, after S Clinton St (across from Union Station) -&gt; Multi-Modal/Rental Car Facility</t>
         </is>
       </c>
     </row>
@@ -1559,17 +1559,17 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>d18 Sat 11:50 Four Winds Casino Shuttle (Chinatown)</t>
+          <t>d18 Sat 09:08 Metra</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>35th &amp; State St (Four Winds shuttle)</t>
+          <t>Kenosha</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Four Winds Casino New Buffalo MI (shuttle)</t>
+          <t>Chicago OTC</t>
         </is>
       </c>
       <c r="E41" s="3" t="n">
@@ -1577,7 +1577,7 @@
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>d18 Sat 13:50 Four Winds Casino Shuttle (Chinatown): 35th &amp; State St (Four Winds shuttle) -&gt; Four Winds Casino New Buffalo MI (shuttle)</t>
+          <t>d18 Sat 09:30 Wisconsin Coach Lines: Metro Train Station - 13th Avenue and 54th Street -&gt; Mitchell Airport</t>
         </is>
       </c>
     </row>
@@ -1587,17 +1587,17 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>d18 Sat 15:00 Four Winds Casino Shuttle (Chinatown)</t>
+          <t>d18 Sat 11:07 Chicago Transit Authority</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Four Winds Casino New Buffalo MI (shuttle)</t>
+          <t>Clinton-Green</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>2734 S. Wentworth Bus Depot (Four Winds shuttle)</t>
+          <t>35-Bronzeville-IIT</t>
         </is>
       </c>
       <c r="E42" s="3" t="n">
@@ -1605,7 +1605,7 @@
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>d18 Sat 17:00 Four Winds Casino Shuttle (Chinatown): Four Winds Casino New Buffalo MI (shuttle) -&gt; 2734 S. Wentworth Bus Depot (Four Winds shuttle)</t>
+          <t>d18 Sat 11:17 Chicago Transit Authority: Clinton-Green -&gt; 35-Bronzeville-IIT</t>
         </is>
       </c>
     </row>
@@ -1615,25 +1615,25 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>d18 Sat 21:15 Jefferson Lines</t>
+          <t>d18 Sat 11:50 Four Winds Casino Shuttle (Chinatown)</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Chicago Bus Station</t>
+          <t>35th &amp; State St (Four Winds shuttle)</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Omaha</t>
-        </is>
-      </c>
-      <c r="E43" s="2" t="n">
-        <v>24</v>
+          <t>Four Winds Casino New Buffalo MI (shuttle)</t>
+        </is>
+      </c>
+      <c r="E43" s="3" t="n">
+        <v>0</v>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>d19 Sun 12:25 Greyhound-us: Chicago Bus Station -&gt; Omaha, NE</t>
+          <t>d18 Sat 13:50 Four Winds Casino Shuttle (Chinatown): 35th &amp; State St (Four Winds shuttle) -&gt; Four Winds Casino New Buffalo MI (shuttle)</t>
         </is>
       </c>
     </row>
@@ -1643,25 +1643,25 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>d19 Sun 06:15 Jefferson Lines</t>
+          <t>d18 Sat 15:00 Four Winds Casino Shuttle (Chinatown)</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Omaha</t>
+          <t>Four Winds Casino New Buffalo MI (shuttle)</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Sioux Falls</t>
-        </is>
-      </c>
-      <c r="E44" s="2" t="n">
-        <v>24</v>
+          <t>Archer and Wentworth (Four Winds shuttle)</t>
+        </is>
+      </c>
+      <c r="E44" s="3" t="n">
+        <v>0</v>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>d20 Mon 06:15 Jefferson Lines: Omaha -&gt; Sioux Falls</t>
+          <t>d18 Sat 17:00 Four Winds Casino Shuttle (Chinatown): Four Winds Casino New Buffalo MI (shuttle) -&gt; Archer and Wentworth (Four Winds shuttle)</t>
         </is>
       </c>
     </row>
@@ -1671,23 +1671,107 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
+          <t>d18 Sat 15:47 Chicago Transit Authority</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Cermak-Chinatown</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Harrison</t>
+        </is>
+      </c>
+      <c r="E45" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>d18 Sat 15:53 Chicago Transit Authority: Cermak-Chinatown -&gt; Monroe-Red</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="n">
+        <v>44</v>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>d18 Sat 21:15 Jefferson Lines</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Chicago Bus Station</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Omaha</t>
+        </is>
+      </c>
+      <c r="E46" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>d19 Sun 12:25 Greyhound-us: Chicago Bus Station -&gt; Omaha, NE</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="n">
+        <v>45</v>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>d19 Sun 06:15 Jefferson Lines</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Omaha</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Sioux Falls</t>
+        </is>
+      </c>
+      <c r="E47" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>d20 Mon 06:15 Jefferson Lines: Omaha -&gt; Sioux Falls</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="n">
+        <v>46</v>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
           <t>d19 Sun 10:00 Jefferson Lines</t>
         </is>
       </c>
-      <c r="C45" t="inlineStr">
+      <c r="C48" t="inlineStr">
         <is>
           <t>Sioux Falls</t>
         </is>
       </c>
-      <c r="D45" t="inlineStr">
+      <c r="D48" t="inlineStr">
         <is>
           <t>Fargo</t>
         </is>
       </c>
-      <c r="E45" s="4" t="n">
-        <v>8.199999999999999</v>
-      </c>
-      <c r="F45" t="inlineStr">
+      <c r="E48" s="4" t="n">
+        <v>7.8</v>
+      </c>
+      <c r="F48" t="inlineStr">
         <is>
           <t>d19 Sun 10:30 Jefferson Lines: Sioux Falls -&gt; Minneapolis</t>
         </is>
@@ -1704,7 +1788,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F41"/>
+  <dimension ref="A1:F43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -1984,17 +2068,17 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>d4 Thu 04:45 Salt Lake Express</t>
+          <t>d4 Thu 03:57 Utah Transit Authority</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Salt Lake City (Airport)</t>
+          <t>Salt Lake Central Station (Bay A)</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Saint George (Bluff St Office)</t>
+          <t>400 S / 300 W (EB)</t>
         </is>
       </c>
       <c r="E11" s="3" t="n">
@@ -2002,7 +2086,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>d4 Thu 06:00 Salt Lake Express: Salt Lake City (Airport) -&gt; Las Vegas (Airport)</t>
+          <t>d4 Thu 04:13 Utah Transit Authority: Salt Lake Central Station (Bay A) -&gt; 200 S / West Temple (EB)</t>
         </is>
       </c>
     </row>
@@ -2012,17 +2096,17 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>d4 Thu 10:30 Salt Lake Express</t>
+          <t>d4 Thu 04:48 Utah Transit Authority</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Saint George (Bluff St Office)</t>
+          <t>900 South Station</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Las Vegas (Airport)</t>
+          <t>Airport Station</t>
         </is>
       </c>
       <c r="E12" s="3" t="n">
@@ -2030,7 +2114,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>d4 Thu 12:00 Salt Lake Express: Saint George (Bluff St Office) -&gt; Las Vegas (Airport)</t>
+          <t>d4 Thu 05:03 Utah Transit Authority: 900 South Station -&gt; Airport Station</t>
         </is>
       </c>
     </row>
@@ -2040,17 +2124,17 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>d4 Thu 14:00 Greyhound-us</t>
+          <t>d4 Thu 06:00 St George Shuttle</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Las Vegas Bus Terminal</t>
+          <t>Salt Lake City (Airport)</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>San Bernardino Depot</t>
+          <t>Las Vegas (Airport)</t>
         </is>
       </c>
       <c r="E13" s="3" t="n">
@@ -2058,7 +2142,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>d4 Thu 15:15 702 Shuttles: Las Vegas Dean Martin Blue Diamond (702 Shuttles) -&gt; Victorville 15445 Palmdale Rd (702 Shuttles)</t>
+          <t>d4 Thu 06:45 Salt Lake Express: Salt Lake City (Airport) -&gt; Saint George (Bluff St Office)</t>
         </is>
       </c>
     </row>
@@ -2068,25 +2152,25 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>d4 Thu 18:43 Amtrak</t>
+          <t xml:space="preserve">d4 Thu 13:18 Regional Transportation Commission of Southern Nevada </t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>San Bernardino</t>
+          <t>Harry Reid Intl Airport Zero Level</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Newton</t>
-        </is>
-      </c>
-      <c r="E14" s="2" t="n">
-        <v>24</v>
+          <t>NB Maryland before Charleston</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="n">
+        <v>0</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>wait 1 day(s) and catch the same bus, then continue</t>
+          <t>d4 Thu 13:30 Regional Transportation Commission of Southern Nevada : Harry Reid Intl Airport Zero Level -&gt; NB Maryland before Charleston</t>
         </is>
       </c>
     </row>
@@ -2096,25 +2180,25 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>d6 Sat 03:00 BeeLine Express-Village Travel</t>
+          <t xml:space="preserve">d4 Thu 14:08 Regional Transportation Commission of Southern Nevada </t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Newton (Amtrak)</t>
+          <t>EB Bonneville before 10th</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Oklahoma City</t>
-        </is>
-      </c>
-      <c r="E15" s="2" t="n">
-        <v>24</v>
+          <t>EB Searles after 21st</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="n">
+        <v>0</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>d6 Sat 05:30 BeeLine Express-Village Travel: Newton (Amtrak) -&gt; Wichita</t>
+          <t>d4 Thu 15:05 FlixBus-us: Las Vegas Downtown (1st St) -&gt; Barstow Station</t>
         </is>
       </c>
     </row>
@@ -2124,25 +2208,25 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>d6 Sat 06:55 Greyhound-us</t>
+          <t>d4 Thu 15:00 702 Shuttles</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Oklahoma City Bus Station</t>
+          <t>Las Vegas 1404 N Eastern Ave (702 Shuttles)</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Dallas Bus Station</t>
-        </is>
-      </c>
-      <c r="E16" s="3" t="n">
-        <v>0</v>
+          <t>Barstow East Main St 1611 (702 Shuttles)</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="n">
+        <v>24</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>d6 Sat 08:35 FlixBus-us: Oklahoma City Bus Station -&gt; Dallas Bus Station</t>
+          <t>wait 1 day(s) and catch the same bus, then continue</t>
         </is>
       </c>
     </row>
@@ -2152,25 +2236,25 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>d6 Sat 11:30 FlixBus-us</t>
+          <t>d4 Thu 20:47 Amtrak</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Dallas Bus Station</t>
+          <t>Barstow</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Downtown Houston (Gray St.)</t>
-        </is>
-      </c>
-      <c r="E17" s="3" t="n">
-        <v>0</v>
+          <t>Newton</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="n">
+        <v>24</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>d6 Sat 11:50 DALLAS AREA RAPID TRANSIT: BACHMAN STATION -&gt; AKARD STATION</t>
+          <t>wait 1 day(s) and catch the same bus, then continue</t>
         </is>
       </c>
     </row>
@@ -2180,25 +2264,25 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>d6 Sat 16:48 Metropolitan Transit Authority of Harris County</t>
+          <t>d6 Sat 03:00 BeeLine Express-Village Travel</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Theater District Rusk EB</t>
+          <t>Newton (Amtrak)</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Magnolia Park Transit Center EB</t>
-        </is>
-      </c>
-      <c r="E18" s="3" t="n">
-        <v>0</v>
+          <t>Oklahoma City</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="n">
+        <v>24</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>d6 Sat 17:06 Metropolitan Transit Authority of Harris County: Theater District Rusk EB -&gt; Magnolia Park Transit Center EB</t>
+          <t>d6 Sat 05:30 BeeLine Express-Village Travel: Newton (Amtrak) -&gt; Wichita</t>
         </is>
       </c>
     </row>
@@ -2208,25 +2292,25 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>d6 Sat 18:35 Greyhound-us</t>
+          <t>d6 Sat 06:55 Greyhound-us</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Houston Bus Station (Greyhound)</t>
+          <t>Oklahoma City Bus Station</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Tallahassee (CK Steele Bus Plaza)</t>
-        </is>
-      </c>
-      <c r="E19" s="2" t="n">
-        <v>24</v>
+          <t>Dallas Bus Station</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="n">
+        <v>0</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>d6 Sat 22:00 Greyhound-us: Houston Bus Station (Greyhound) -&gt; Mobile Bus Station</t>
+          <t>d6 Sat 08:35 FlixBus-us: Oklahoma City Bus Station -&gt; Dallas Bus Station</t>
         </is>
       </c>
     </row>
@@ -2236,25 +2320,25 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>d7 Sun 11:25 Greyhound-us</t>
+          <t>d6 Sat 11:30 FlixBus-us</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Tallahassee (CK Steele Bus Plaza)</t>
+          <t>Dallas Bus Station</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Jacksonville (Downtown)</t>
-        </is>
-      </c>
-      <c r="E20" s="2" t="n">
-        <v>24</v>
+          <t>Downtown Houston (Gray St.)</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="n">
+        <v>0</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>d7 Sun 17:10 Greyhound-us: Tallahassee (CK Steele Bus Plaza) -&gt; Jacksonville (Downtown)</t>
+          <t>d6 Sat 11:50 DALLAS AREA RAPID TRANSIT: BACHMAN STATION -&gt; AKARD STATION</t>
         </is>
       </c>
     </row>
@@ -2264,17 +2348,17 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>d7 Sun 15:00 Jacksonville Transportation Authority</t>
+          <t>d6 Sat 16:48 Metropolitan Transit Authority of Harris County</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>JRTC Bay H</t>
+          <t>Theater District Rusk EB</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Amtrak Station</t>
+          <t>Magnolia Park Transit Center EB</t>
         </is>
       </c>
       <c r="E21" s="3" t="n">
@@ -2282,7 +2366,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>d7 Sun 16:11 Amtrak: Jacksonville -&gt; Washington Union Station</t>
+          <t>d6 Sat 17:06 Metropolitan Transit Authority of Harris County: Theater District Rusk EB -&gt; Magnolia Park Transit Center EB</t>
         </is>
       </c>
     </row>
@@ -2292,17 +2376,17 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>d7 Sun 16:11 Amtrak</t>
+          <t>d6 Sat 18:35 Greyhound-us</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Jacksonville</t>
+          <t>Houston Bus Station (Greyhound)</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Washington Union Station</t>
+          <t>Tallahassee (CK Steele Bus Plaza)</t>
         </is>
       </c>
       <c r="E22" s="2" t="n">
@@ -2310,7 +2394,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>wait 1 day(s) and catch the same bus, then continue</t>
+          <t>d6 Sat 22:00 Greyhound-us: Houston Bus Station (Greyhound) -&gt; Mobile Bus Station</t>
         </is>
       </c>
     </row>
@@ -2320,17 +2404,17 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>d8 Mon 06:50 Amtrak</t>
+          <t>d7 Sun 11:25 Greyhound-us</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Washington Union Station</t>
+          <t>Tallahassee (CK Steele Bus Plaza)</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Boston</t>
+          <t>Jacksonville (Downtown)</t>
         </is>
       </c>
       <c r="E23" s="2" t="n">
@@ -2338,7 +2422,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>wait 1 day(s) and catch the same bus, then continue</t>
+          <t>d7 Sun 17:10 Greyhound-us: Tallahassee (CK Steele Bus Plaza) -&gt; Jacksonville (Downtown)</t>
         </is>
       </c>
     </row>
@@ -2348,17 +2432,17 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>d8 Mon 14:15 Concord Coach Lines</t>
+          <t>d7 Sun 15:00 Jacksonville Transportation Authority</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Boston South Station</t>
+          <t>JRTC Bay H</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Portland, ME</t>
+          <t>Amtrak Station</t>
         </is>
       </c>
       <c r="E24" s="3" t="n">
@@ -2366,7 +2450,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>d8 Mon 15:15 Concord Coach Lines: Boston South Station -&gt; Portland, ME</t>
+          <t>d7 Sun 18:30 FlixBus-us: Jacksonville (Downtown) -&gt; Washington Union Station</t>
         </is>
       </c>
     </row>
@@ -2376,17 +2460,17 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>d8 Mon 16:45 Concord Coach Lines</t>
+          <t>d7 Sun 16:11 Amtrak</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Portland, ME</t>
+          <t>Jacksonville</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Boston South Station</t>
+          <t>Washington Union Station</t>
         </is>
       </c>
       <c r="E25" s="3" t="n">
@@ -2394,7 +2478,7 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>d8 Mon 18:00 Concord Coach Lines: Portland, ME -&gt; Boston South Station</t>
+          <t>d7 Sun 16:27 Jacksonville Transportation Authority: Amtrak Station -&gt; 5001 Soutel Dr</t>
         </is>
       </c>
     </row>
@@ -2404,25 +2488,25 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>d8 Mon 19:30 Dartmouth Coach</t>
+          <t>d8 Mon 06:50 Amtrak</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Boston South Station</t>
+          <t>Washington Union Station</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Hanover (Hanover Inn)</t>
-        </is>
-      </c>
-      <c r="E26" s="3" t="n">
-        <v>0</v>
+          <t>Boston</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="n">
+        <v>24</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>d8 Mon 21:30 Dartmouth Coach: Boston South Station -&gt; Hanover (Hanover Inn)</t>
+          <t>wait 1 day(s) and catch the same bus, then continue</t>
         </is>
       </c>
     </row>
@@ -2432,25 +2516,25 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>d9 Tue 03:00 Dartmouth Coach</t>
+          <t>d8 Mon 14:15 Concord Coach Lines</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Hanover (Hanover Inn)</t>
+          <t>Boston South Station</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Boston South Station</t>
-        </is>
-      </c>
-      <c r="E27" s="2" t="n">
-        <v>24</v>
+          <t>Portland, ME</t>
+        </is>
+      </c>
+      <c r="E27" s="3" t="n">
+        <v>0</v>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>d9 Tue 04:35 Greyhound-us: White River Junction Bus Station -&gt; Boston (South Station)</t>
+          <t>d8 Mon 15:15 Concord Coach Lines: Boston South Station -&gt; Portland, ME</t>
         </is>
       </c>
     </row>
@@ -2460,17 +2544,17 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>d9 Tue 07:00 Amtrak</t>
+          <t>d8 Mon 16:45 Concord Coach Lines</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Boston</t>
+          <t>Portland, ME</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Washington Union Station</t>
+          <t>Boston South Station</t>
         </is>
       </c>
       <c r="E28" s="3" t="n">
@@ -2478,7 +2562,7 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>d9 Tue 07:15 FlixBus-us: Boston (South Station) -&gt; New York Midtown (31st St &amp; 8th Ave)</t>
+          <t>d8 Mon 18:00 Concord Coach Lines: Portland, ME -&gt; Boston South Station</t>
         </is>
       </c>
     </row>
@@ -2488,25 +2572,25 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>d9 Tue 15:57 Amtrak</t>
+          <t>d8 Mon 19:30 Dartmouth Coach</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Washington Union Station</t>
+          <t>Boston South Station</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Toledo</t>
-        </is>
-      </c>
-      <c r="E29" s="2" t="n">
-        <v>24</v>
+          <t>Hanover (Hanover Inn)</t>
+        </is>
+      </c>
+      <c r="E29" s="3" t="n">
+        <v>0</v>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>d9 Tue 17:50 Greyhound-us: Washington Union Station -&gt; Pittsburgh Intermodal Station</t>
+          <t>d8 Mon 21:30 Dartmouth Coach: Boston South Station -&gt; Hanover (Hanover Inn)</t>
         </is>
       </c>
     </row>
@@ -2516,25 +2600,25 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>d10 Wed 06:30 Amtrak Chartered Vehicle</t>
+          <t>d9 Tue 03:00 Dartmouth Coach</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Toledo</t>
+          <t>Hanover (Hanover Inn)</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Detroit</t>
-        </is>
-      </c>
-      <c r="E30" s="4" t="n">
-        <v>8.1</v>
+          <t>Boston South Station</t>
+        </is>
+      </c>
+      <c r="E30" s="3" t="n">
+        <v>0</v>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>d10 Wed 07:55 Greyhound-us: Toledo Bus Stop -&gt; Detroit Bus Station</t>
+          <t>d9 Tue 06:30 Dartmouth Coach: Hanover (Hanover Inn) -&gt; Dartmouth Coach NYC (150 E 42nd St)</t>
         </is>
       </c>
     </row>
@@ -2544,17 +2628,17 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>d10 Wed 07:44 Detroit Department of Transportation</t>
+          <t>d9 Tue 07:00 Amtrak</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Woodward &amp; Baltimore</t>
+          <t>Boston</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Woodward &amp; State Fair</t>
+          <t>Washington Union Station</t>
         </is>
       </c>
       <c r="E31" s="3" t="n">
@@ -2562,7 +2646,7 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>d10 Wed 09:35 Amtrak: Detroit -&gt; Chicago Union Station</t>
+          <t>d9 Tue 07:15 FlixBus-us: Boston (South Station) -&gt; New York Midtown (31st St &amp; 8th Ave)</t>
         </is>
       </c>
     </row>
@@ -2572,25 +2656,25 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>d10 Wed 09:12 Amtrak</t>
+          <t>d9 Tue 15:57 Amtrak</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Royal Oak Amtrak</t>
+          <t>Washington Union Station</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Chicago Union Station</t>
+          <t>Toledo</t>
         </is>
       </c>
       <c r="E32" s="2" t="n">
-        <v>21.4</v>
+        <v>24</v>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>d10 Wed 10:12 Detroit Department of Transportation: Jason Hargrove Transit Center - Bay 4 -&gt; Rosa Parks Transit Center - Bay 15</t>
+          <t>d9 Tue 17:50 Greyhound-us: Washington Union Station -&gt; Pittsburgh Intermodal Station</t>
         </is>
       </c>
     </row>
@@ -2600,25 +2684,25 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>d10 Wed 14:10 Van Galder (Coach USA)</t>
+          <t>d10 Wed 06:30 Amtrak Chartered Vehicle</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>W Jackson Blvd, after S Clinton St (across from Union Station)</t>
+          <t>Toledo</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Multi-Modal/Rental Car Facility</t>
-        </is>
-      </c>
-      <c r="E33" s="3" t="n">
-        <v>0</v>
+          <t>Detroit</t>
+        </is>
+      </c>
+      <c r="E33" s="4" t="n">
+        <v>8.1</v>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>d10 Wed 15:05 Amtrak: Chicago Union Station -&gt; Milwaukee</t>
+          <t>d10 Wed 07:55 Greyhound-us: Toledo Bus Stop -&gt; Detroit Bus Station</t>
         </is>
       </c>
     </row>
@@ -2628,25 +2712,25 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>d10 Wed 15:30 Wisconsin Coach Lines</t>
+          <t>d10 Wed 09:35 Amtrak</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Multi-Modal/Rental Car Facility</t>
+          <t>Detroit</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Kenosha Brat Stop</t>
-        </is>
-      </c>
-      <c r="E34" s="3" t="n">
-        <v>0</v>
+          <t>Chicago Union Station</t>
+        </is>
+      </c>
+      <c r="E34" s="4" t="n">
+        <v>8.1</v>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>d10 Wed 16:30 Wisconsin Coach Lines: Multi-Modal/Rental Car Facility -&gt; Kenosha Brat Stop</t>
+          <t>d10 Wed 09:49 Detroit Department of Transportation: Cass &amp; Milwaukee -&gt; Washington &amp; Michigan</t>
         </is>
       </c>
     </row>
@@ -2656,17 +2740,17 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>d10 Wed 16:45 Wisconsin Coach Lines</t>
+          <t>d10 Wed 14:10 Van Galder (Coach USA)</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Kenosha Brat Stop</t>
+          <t>W Jackson Blvd, after S Clinton St (across from Union Station)</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>O'Hare International Airport - Terminal 2 Departures</t>
+          <t>Multi-Modal/Rental Car Facility</t>
         </is>
       </c>
       <c r="E35" s="3" t="n">
@@ -2674,7 +2758,7 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>d10 Wed 17:45 Wisconsin Coach Lines: Kenosha Brat Stop -&gt; O'Hare International Airport - Terminal 1 Departures</t>
+          <t>d10 Wed 15:05 Amtrak: Chicago Union Station -&gt; Milwaukee</t>
         </is>
       </c>
     </row>
@@ -2684,17 +2768,17 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>d10 Wed 17:37 Chicago Transit Authority</t>
+          <t>d10 Wed 15:30 Wisconsin Coach Lines</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>O'Hare</t>
+          <t>Multi-Modal/Rental Car Facility</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Clinton-Blue</t>
+          <t>Kenosha Brat Stop</t>
         </is>
       </c>
       <c r="E36" s="3" t="n">
@@ -2702,7 +2786,7 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>d10 Wed 17:45 Chicago Transit Authority: O'Hare -&gt; Clinton-Blue</t>
+          <t>d10 Wed 16:30 Wisconsin Coach Lines: Multi-Modal/Rental Car Facility -&gt; Kenosha Brat Stop</t>
         </is>
       </c>
     </row>
@@ -2712,25 +2796,25 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>d10 Wed 20:05 Amtrak</t>
+          <t>d10 Wed 16:45 Wisconsin Coach Lines</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Chicago Union Station</t>
+          <t>Kenosha Brat Stop</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Memphis</t>
-        </is>
-      </c>
-      <c r="E37" s="4" t="n">
-        <v>8.1</v>
+          <t>O'Hare International Airport - Terminal 2 Departures</t>
+        </is>
+      </c>
+      <c r="E37" s="3" t="n">
+        <v>0</v>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>d10 Wed 22:50 Greyhound-us: Chicago Bus Station -&gt; Nashville Bus Station</t>
+          <t>d10 Wed 17:45 Wisconsin Coach Lines: Kenosha Brat Stop -&gt; O'Hare International Airport - Terminal 1 Departures</t>
         </is>
       </c>
     </row>
@@ -2740,17 +2824,17 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>d11 Thu 06:55 On foot (Big River Crossing, open 06:00-22:00)</t>
+          <t>d10 Wed 17:37 Chicago Transit Authority</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Memphis</t>
+          <t>O'Hare</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Arkansas line on Big River Crossing (on foot from Memphis Amtrak)</t>
+          <t>Clinton-Blue</t>
         </is>
       </c>
       <c r="E38" s="3" t="n">
@@ -2758,7 +2842,7 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>d11 Thu 07:05 On foot (Big River Crossing, open 06:00-22:00): Memphis -&gt; Arkansas line on Big River Crossing (on foot from Memphis Amtrak)</t>
+          <t>d10 Wed 17:45 Chicago Transit Authority: O'Hare -&gt; Clinton-Blue</t>
         </is>
       </c>
     </row>
@@ -2768,12 +2852,12 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>d11 Thu 07:40 On foot (Big River Crossing, open 06:00-22:00)</t>
+          <t>d10 Wed 20:05 Amtrak</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Arkansas line on Big River Crossing (on foot from Memphis Amtrak)</t>
+          <t>Chicago Union Station</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -2781,12 +2865,12 @@
           <t>Memphis</t>
         </is>
       </c>
-      <c r="E39" s="3" t="n">
-        <v>0</v>
+      <c r="E39" s="4" t="n">
+        <v>8.1</v>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>d11 Thu 07:50 On foot (Big River Crossing, open 06:00-22:00): Arkansas line on Big River Crossing (on foot from Memphis Amtrak) -&gt; Memphis</t>
+          <t>d10 Wed 22:50 Greyhound-us: Chicago Bus Station -&gt; Nashville Bus Station</t>
         </is>
       </c>
     </row>
@@ -2796,17 +2880,17 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>d11 Thu 08:43 MATA</t>
+          <t>d11 Thu 06:55 On foot (Big River Crossing, open 06:00-22:00)</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>UNION AVENUE at 3RD STREET</t>
+          <t>Memphis</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>WILLIAM HUDSON TRANSIT CENTER</t>
+          <t>Arkansas line on Big River Crossing (on foot from Memphis Amtrak)</t>
         </is>
       </c>
       <c r="E40" s="3" t="n">
@@ -2814,7 +2898,7 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>d11 Thu 08:57 MATA: 3RD STREET at UNION AVENUE -&gt; WILLIAM HUDSON TRANSIT CENTER</t>
+          <t>d11 Thu 07:05 On foot (Big River Crossing, open 06:00-22:00): Memphis -&gt; Arkansas line on Big River Crossing (on foot from Memphis Amtrak)</t>
         </is>
       </c>
     </row>
@@ -2824,23 +2908,79 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
+          <t>d11 Thu 07:40 On foot (Big River Crossing, open 06:00-22:00)</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Arkansas line on Big River Crossing (on foot from Memphis Amtrak)</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Memphis</t>
+        </is>
+      </c>
+      <c r="E41" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>d11 Thu 07:50 On foot (Big River Crossing, open 06:00-22:00): Arkansas line on Big River Crossing (on foot from Memphis Amtrak) -&gt; Memphis</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="n">
+        <v>40</v>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>d11 Thu 08:43 MATA</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>UNION AVENUE at 3RD STREET</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>WILLIAM HUDSON TRANSIT CENTER</t>
+        </is>
+      </c>
+      <c r="E42" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>d11 Thu 08:57 MATA: 3RD STREET at UNION AVENUE -&gt; WILLIAM HUDSON TRANSIT CENTER</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>41</v>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
           <t>d11 Thu 09:15 MATA</t>
         </is>
       </c>
-      <c r="C41" t="inlineStr">
+      <c r="C43" t="inlineStr">
         <is>
           <t>WILLIAM HUDSON TRANSIT CENTER</t>
         </is>
       </c>
-      <c r="D41" t="inlineStr">
+      <c r="D43" t="inlineStr">
         <is>
           <t>IRS</t>
         </is>
       </c>
-      <c r="E41" s="3" t="n">
+      <c r="E43" s="3" t="n">
         <v>1.1</v>
       </c>
-      <c r="F41" t="inlineStr">
+      <c r="F43" t="inlineStr">
         <is>
           <t>d11 Thu 09:45 MATA: WILLIAM HUDSON TRANSIT CENTER -&gt; JEFFERSON AVENUE at MONTGOMERY STREET</t>
         </is>
@@ -2857,7 +2997,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F39"/>
+  <dimension ref="A1:F42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -2871,7 +3011,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Control: 237.66 h. Miss each ride by one minute and replay the rest.</t>
+          <t>Control: 237.49 h from the first bus. Miss each ride by one minute and replay the rest.</t>
         </is>
       </c>
     </row>
@@ -3063,7 +3203,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>AIRWAYS BOULEVARD at HOLMES ROAD</t>
+          <t>HOLMES ROAD at HORNSBY DRIVE</t>
         </is>
       </c>
       <c r="E8" s="2" t="n">
@@ -3081,25 +3221,25 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>d10 Fri 08:20 MATA</t>
+          <t>d10 Fri 08:08 MATA</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>AIRWAYS BOULEVARD at HOLMES ROAD</t>
+          <t>HOLMES RD at HORNSBY DR</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>HOLMES ROAD at HORNSBY DRIVE</t>
-        </is>
-      </c>
-      <c r="E9" s="3" t="n">
-        <v>0</v>
+          <t>AIRWAYS TRANSIT CENTER</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="n">
+        <v>24</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>d10 Fri 09:30 FlixBus-us: Memphis Bus Station -&gt; St Louis Bus Station</t>
+          <t>d10 Fri 08:21 MATA: HOLMES ROAD at HORNSBY DRIVE -&gt; ELVIS PRESLEY BLVD at SPRINGBROOK AVENUE</t>
         </is>
       </c>
     </row>
@@ -3183,7 +3323,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>d11 Sat 01:30 Jefferson Lines: Kansas City Bus Station -&gt; Omaha</t>
+          <t>d10 Fri 21:44 Kansas City Area Transportation Authority: ON MAIN AT 27TH STREET NORTHBOUND NEARSIDE -&gt; EAST VILLAGE - BAY B</t>
         </is>
       </c>
     </row>
@@ -3295,7 +3435,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>d12 Sun 03:29 Amtrak: Fargo Amtrak Station -&gt; St. Paul-Minneapolis</t>
+          <t>d12 Sun 10:35 Jefferson Lines: Fargo -&gt; Brainerd</t>
         </is>
       </c>
     </row>
@@ -3473,17 +3613,17 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>d14 Tue 04:45 Salt Lake Express</t>
+          <t>d14 Tue 03:57 Utah Transit Authority</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Salt Lake City (Airport)</t>
+          <t>Salt Lake Central Station (Bay A)</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Saint George (Bluff St Office)</t>
+          <t>400 S / 300 W (EB)</t>
         </is>
       </c>
       <c r="E23" s="3" t="n">
@@ -3491,7 +3631,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>d14 Tue 06:00 Salt Lake Express: Salt Lake City (Airport) -&gt; Saint George (Bluff St Office)</t>
+          <t>d14 Tue 04:13 Utah Transit Authority: Salt Lake Central Station (Bay A) -&gt; 200 S / West Temple (EB)</t>
         </is>
       </c>
     </row>
@@ -3501,17 +3641,17 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>d14 Tue 10:30 Salt Lake Express</t>
+          <t>d14 Tue 04:48 Utah Transit Authority</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Saint George (Bluff St Office)</t>
+          <t>900 South Station</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Las Vegas (Airport)</t>
+          <t>Airport Station</t>
         </is>
       </c>
       <c r="E24" s="3" t="n">
@@ -3519,7 +3659,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>d14 Tue 12:15 Salt Lake Express: Saint George (Shop) -&gt; Las Vegas (Airport)</t>
+          <t>d14 Tue 05:03 Utah Transit Authority: 900 South Station -&gt; Airport Station</t>
         </is>
       </c>
     </row>
@@ -3529,17 +3669,17 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>d14 Tue 14:00 Greyhound-us</t>
+          <t>d14 Tue 06:00 St George Shuttle</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Las Vegas Bus Terminal</t>
+          <t>Salt Lake City (Airport)</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>San Bernardino Depot</t>
+          <t>Las Vegas (Airport)</t>
         </is>
       </c>
       <c r="E25" s="3" t="n">
@@ -3547,7 +3687,7 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>d14 Tue 15:15 702 Shuttles: Las Vegas Dean Martin Blue Diamond (702 Shuttles) -&gt; Victorville 15445 Palmdale Rd (702 Shuttles)</t>
+          <t>d14 Tue 06:45 Salt Lake Express: Salt Lake City (Airport) -&gt; Saint George (Bluff St Office)</t>
         </is>
       </c>
     </row>
@@ -3557,25 +3697,25 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>d14 Tue 18:43 Amtrak</t>
+          <t xml:space="preserve">d14 Tue 13:18 Regional Transportation Commission of Southern Nevada </t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>San Bernardino</t>
+          <t>Harry Reid Intl Airport Zero Level</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Newton</t>
-        </is>
-      </c>
-      <c r="E26" s="2" t="n">
-        <v>24</v>
+          <t>NB Maryland before Charleston</t>
+        </is>
+      </c>
+      <c r="E26" s="3" t="n">
+        <v>0</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>wait 1 day(s) and catch the same bus, then continue</t>
+          <t>d14 Tue 13:30 Regional Transportation Commission of Southern Nevada : Harry Reid Intl Airport Zero Level -&gt; NB Maryland before Charleston</t>
         </is>
       </c>
     </row>
@@ -3585,25 +3725,25 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>d16 Thu 03:00 BeeLine Express-Village Travel</t>
+          <t xml:space="preserve">d14 Tue 14:08 Regional Transportation Commission of Southern Nevada </t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Newton (Amtrak)</t>
+          <t>EB Bonneville before 10th</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Oklahoma City</t>
-        </is>
-      </c>
-      <c r="E27" s="2" t="n">
-        <v>24</v>
+          <t>EB Searles after 21st</t>
+        </is>
+      </c>
+      <c r="E27" s="3" t="n">
+        <v>0</v>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>d16 Thu 05:30 BeeLine Express-Village Travel: Newton (Amtrak) -&gt; Wichita</t>
+          <t>d14 Tue 15:05 FlixBus-us: Las Vegas Downtown (1st St) -&gt; Barstow Station</t>
         </is>
       </c>
     </row>
@@ -3613,25 +3753,25 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>d16 Thu 06:55 Greyhound-us</t>
+          <t>d14 Tue 15:00 702 Shuttles</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Oklahoma City Bus Station</t>
+          <t>Las Vegas 1404 N Eastern Ave (702 Shuttles)</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Dallas Bus Station</t>
-        </is>
-      </c>
-      <c r="E28" s="3" t="n">
-        <v>0</v>
+          <t>Barstow East Main St 1611 (702 Shuttles)</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="n">
+        <v>24</v>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>d16 Thu 10:15 Vonlane: Oklahoma City Omni (Vonlane) -&gt; Dallas DoubleTree Love Field (Vonlane)</t>
+          <t>wait 1 day(s) and catch the same bus, then continue</t>
         </is>
       </c>
     </row>
@@ -3641,25 +3781,25 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>d16 Thu 11:25 DALLAS AREA RAPID TRANSIT</t>
+          <t>d14 Tue 20:47 Amtrak</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>BACHMAN STATION</t>
+          <t>Barstow</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>AKARD STATION</t>
-        </is>
-      </c>
-      <c r="E29" s="3" t="n">
-        <v>0</v>
+          <t>Newton</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="n">
+        <v>24</v>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>d16 Thu 11:45 DALLAS AREA RAPID TRANSIT: BACHMAN STATION -&gt; AKARD STATION</t>
+          <t>wait 1 day(s) and catch the same bus, then continue</t>
         </is>
       </c>
     </row>
@@ -3669,25 +3809,25 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>d16 Thu 12:35 RedCoach</t>
+          <t>d16 Thu 03:00 BeeLine Express-Village Travel</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Dallas 1376 Marilla St (RedCoach)</t>
+          <t>Newton (Amtrak)</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Houston 808 Jefferson St (RedCoach)</t>
-        </is>
-      </c>
-      <c r="E30" s="3" t="n">
-        <v>0</v>
+          <t>Oklahoma City</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="n">
+        <v>24</v>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>d16 Thu 12:58 DALLAS AREA RAPID TRANSIT: AKARD STATION -&gt; BURBANK STATION</t>
+          <t>d16 Thu 05:30 BeeLine Express-Village Travel: Newton (Amtrak) -&gt; Wichita</t>
         </is>
       </c>
     </row>
@@ -3697,17 +3837,17 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>d16 Thu 17:45 FlixBus-us</t>
+          <t>d16 Thu 06:55 Greyhound-us</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Downtown Houston (Gray St.)</t>
+          <t>Oklahoma City Bus Station</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Lake Charles (City Point)</t>
+          <t>Dallas Bus Station</t>
         </is>
       </c>
       <c r="E31" s="3" t="n">
@@ -3715,7 +3855,7 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>d16 Thu 18:03 Metropolitan Transit Authority of Harris County: St Joseph Pkwy @ Louisiana St -&gt; Washington Ave @ Preston St</t>
+          <t>d16 Thu 07:18 EMBARK: NE 4 St @ N Wisconsin Ave -&gt; NW 4 St @ N Broadway Ave</t>
         </is>
       </c>
     </row>
@@ -3725,17 +3865,17 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>d16 Thu 21:10 Greyhound-us</t>
+          <t>d16 Thu 11:25 DALLAS AREA RAPID TRANSIT</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Lake Charles (City Point)</t>
+          <t>BACHMAN STATION</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Tallahassee (CK Steele Bus Plaza)</t>
+          <t>AKARD STATION</t>
         </is>
       </c>
       <c r="E32" s="3" t="n">
@@ -3743,7 +3883,7 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>d16 Thu 22:35 Omnibus Express: Lake Charles -&gt; Lake City</t>
+          <t>d16 Thu 11:45 DALLAS AREA RAPID TRANSIT: BACHMAN STATION -&gt; AKARD STATION</t>
         </is>
       </c>
     </row>
@@ -3753,25 +3893,25 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>d17 Fri 11:25 Greyhound-us</t>
+          <t>d16 Thu 12:35 RedCoach</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Tallahassee (CK Steele Bus Plaza)</t>
+          <t>Dallas 1376 Marilla St (RedCoach)</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Jacksonville (Downtown)</t>
-        </is>
-      </c>
-      <c r="E33" s="4" t="n">
-        <v>16</v>
+          <t>Houston 808 Jefferson St (RedCoach)</t>
+        </is>
+      </c>
+      <c r="E33" s="3" t="n">
+        <v>0</v>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>d17 Fri 17:10 Greyhound-us: Tallahassee (CK Steele Bus Plaza) -&gt; Jacksonville (Downtown)</t>
+          <t>d16 Thu 12:58 DALLAS AREA RAPID TRANSIT: AKARD STATION -&gt; INWOOD/LOVE FIELD STATION</t>
         </is>
       </c>
     </row>
@@ -3781,17 +3921,17 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>d17 Fri 15:00 Jacksonville Transportation Authority</t>
+          <t>d16 Thu 17:45 FlixBus-us</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>JRTC Bay H</t>
+          <t>Downtown Houston (Gray St.)</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Amtrak Station</t>
+          <t>Lake Charles (City Point)</t>
         </is>
       </c>
       <c r="E34" s="3" t="n">
@@ -3799,7 +3939,7 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>d17 Fri 16:11 Amtrak: Jacksonville -&gt; Washington Union Station</t>
+          <t>d16 Thu 18:03 Metropolitan Transit Authority of Harris County: St Joseph Pkwy @ Louisiana St -&gt; Washington Ave @ Preston St</t>
         </is>
       </c>
     </row>
@@ -3809,25 +3949,25 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>d17 Fri 16:11 Amtrak</t>
+          <t>d16 Thu 21:10 Greyhound-us</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Jacksonville</t>
+          <t>Lake Charles (City Point)</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Washington Union Station</t>
-        </is>
-      </c>
-      <c r="E35" s="4" t="n">
-        <v>3.8</v>
+          <t>Tallahassee (CK Steele Bus Plaza)</t>
+        </is>
+      </c>
+      <c r="E35" s="3" t="n">
+        <v>0</v>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>d17 Fri 16:27 Jacksonville Transportation Authority: Amtrak Station -&gt; JRTC Bay H</t>
+          <t>d16 Thu 22:35 Omnibus Express: Lake Charles -&gt; Lake City</t>
         </is>
       </c>
     </row>
@@ -3837,25 +3977,25 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>d18 Sat 06:40 Amtrak</t>
+          <t>d17 Fri 11:25 Greyhound-us</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Washington Union Station</t>
+          <t>Tallahassee (CK Steele Bus Plaza)</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Boston</t>
+          <t>Jacksonville (Downtown)</t>
         </is>
       </c>
       <c r="E36" s="4" t="n">
-        <v>3.8</v>
+        <v>16</v>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>d18 Sat 07:48 Amtrak: Washington Union Station -&gt; Boston</t>
+          <t>d17 Fri 17:10 Greyhound-us: Tallahassee (CK Steele Bus Plaza) -&gt; Jacksonville (Downtown)</t>
         </is>
       </c>
     </row>
@@ -3865,25 +4005,25 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>d18 Sat 14:15 Concord Coach Lines</t>
+          <t>d17 Fri 15:00 Jacksonville Transportation Authority</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Boston South Station</t>
+          <t>JRTC Bay H</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Portland, ME</t>
-        </is>
-      </c>
-      <c r="E37" s="3" t="n">
-        <v>2</v>
+          <t>Amtrak Station</t>
+        </is>
+      </c>
+      <c r="E37" s="4" t="n">
+        <v>3.8</v>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>d18 Sat 15:15 Concord Coach Lines: Boston South Station -&gt; Portland, ME</t>
+          <t>d17 Fri 18:30 FlixBus-us: Jacksonville (Downtown) -&gt; Washington Union Station</t>
         </is>
       </c>
     </row>
@@ -3893,25 +4033,25 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>d18 Sat 16:45 Concord Coach Lines</t>
+          <t>d17 Fri 16:11 Amtrak</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Portland, ME</t>
+          <t>Jacksonville</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Boston South Station</t>
-        </is>
-      </c>
-      <c r="E38" s="3" t="n">
-        <v>2</v>
+          <t>Washington Union Station</t>
+        </is>
+      </c>
+      <c r="E38" s="4" t="n">
+        <v>3.8</v>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>d18 Sat 18:00 Concord Coach Lines: Portland, ME -&gt; Boston South Station</t>
+          <t>d17 Fri 16:27 Jacksonville Transportation Authority: Amtrak Station -&gt; JRTC Bay H</t>
         </is>
       </c>
     </row>
@@ -3921,23 +4061,107 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
+          <t>d18 Sat 06:40 Amtrak</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Washington Union Station</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Boston</t>
+        </is>
+      </c>
+      <c r="E39" s="4" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>d18 Sat 07:48 Amtrak: Washington Union Station -&gt; Boston</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>38</v>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>d18 Sat 14:15 Concord Coach Lines</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Boston South Station</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Portland, ME</t>
+        </is>
+      </c>
+      <c r="E40" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>d18 Sat 15:15 Concord Coach Lines: Boston South Station -&gt; Portland, ME</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>39</v>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>d18 Sat 16:45 Concord Coach Lines</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Portland, ME</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Boston South Station</t>
+        </is>
+      </c>
+      <c r="E41" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>d18 Sat 18:00 Concord Coach Lines: Portland, ME -&gt; Boston South Station</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="n">
+        <v>40</v>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
           <t>d18 Sat 19:30 Dartmouth Coach</t>
         </is>
       </c>
-      <c r="C39" t="inlineStr">
+      <c r="C42" t="inlineStr">
         <is>
           <t>Boston South Station</t>
         </is>
       </c>
-      <c r="D39" t="inlineStr">
+      <c r="D42" t="inlineStr">
         <is>
           <t>Hanover (Hanover Inn)</t>
         </is>
       </c>
-      <c r="E39" s="3" t="n">
+      <c r="E42" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="F39" t="inlineStr">
+      <c r="F42" t="inlineStr">
         <is>
           <t>d18 Sat 21:30 Dartmouth Coach: Boston South Station -&gt; Hanover (Hanover Inn)</t>
         </is>
@@ -3954,7 +4178,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F33"/>
+  <dimension ref="A1:F35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -4028,7 +4252,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>d1 Thu 06:40 Dartmouth Coach: Hanover (Hanover Inn) -&gt; Boston South Station</t>
+          <t>d1 Thu 06:01 Advance Transit: Hartford Town Hall, Opp. -&gt; Hanover Inn</t>
         </is>
       </c>
     </row>
@@ -4056,7 +4280,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>d1 Thu 08:50 Amtrak: Boston -&gt; Portland</t>
+          <t>d1 Thu 08:10 Peter Pan (BZ): Boston (South Station) -&gt; Boston (Logan Airport)</t>
         </is>
       </c>
     </row>
@@ -4196,7 +4420,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>wait 1 day(s) and catch the same bus, then continue</t>
+          <t>d2 Fri 21:05 Greyhound-us: Tallahassee (CK Steele Bus Plaza) -&gt; Orlando Bus Station</t>
         </is>
       </c>
     </row>
@@ -4402,17 +4626,17 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>d6 Tue 09:00 Salt Lake Express</t>
+          <t xml:space="preserve">d6 Tue 06:20 Regional Transportation Commission of Southern Nevada </t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Las Vegas (Airport)</t>
+          <t>SB Valley View after Hacienda</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Saint George (Shop)</t>
+          <t>South Strip Transit Terminal Bay 14</t>
         </is>
       </c>
       <c r="E17" s="3" t="n">
@@ -4420,7 +4644,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>d6 Tue 11:00 Salt Lake Express: Las Vegas (Airport) -&gt; Saint George (Shop)</t>
+          <t>d6 Tue 06:48 Regional Transportation Commission of Southern Nevada : SB Valley View after Tropicana -&gt; South Strip Transit Terminal Bay 14</t>
         </is>
       </c>
     </row>
@@ -4430,25 +4654,25 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>d6 Tue 16:05 Salt Lake Express</t>
+          <t xml:space="preserve">d6 Tue 06:43 Regional Transportation Commission of Southern Nevada </t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Saint George (Shop)</t>
+          <t>South Strip Transit Terminal Bay 18</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Salt Lake City (Airport)</t>
-        </is>
-      </c>
-      <c r="E18" s="2" t="n">
-        <v>24</v>
+          <t>Harry Reid Intl Airport Zero Level</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="n">
+        <v>0</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>d7 Wed 03:35 Salt Lake Express: Saint George (Shop) -&gt; Salt Lake City (Airport)</t>
+          <t>d6 Tue 06:55 Regional Transportation Commission of Southern Nevada : South Strip Transit Terminal Bay 18 -&gt; Harry Reid Intl Airport Zero Level</t>
         </is>
       </c>
     </row>
@@ -4458,25 +4682,25 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>d6 Tue 22:30 Salt Lake Express</t>
+          <t>d6 Tue 08:00 St George Shuttle</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Salt Lake City (Airport)</t>
+          <t>Las Vegas (Airport)</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Pocatello (Transit Depot)</t>
-        </is>
-      </c>
-      <c r="E19" s="4" t="n">
-        <v>18.5</v>
+          <t>Saint George (Bluff St Office)</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="n">
+        <v>0</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>d6 Tue 22:39 Utah Transit Authority: Airport Station -&gt; North Temple Bridge/Guadalupe</t>
+          <t>d6 Tue 09:00 Salt Lake Express: Las Vegas (Airport) -&gt; Saint George (Bluff St Office)</t>
         </is>
       </c>
     </row>
@@ -4486,25 +4710,25 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>d7 Wed 03:40 Salt Lake Express</t>
+          <t>d6 Tue 12:15 St George Shuttle</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Pocatello (Transit Depot)</t>
+          <t>Saint George (Bluff St Office)</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Boise (Airport)</t>
-        </is>
-      </c>
-      <c r="E20" s="2" t="n">
-        <v>24</v>
+          <t>Salt Lake City (Airport)</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="n">
+        <v>0</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>d7 Wed 13:25 Salt Lake Express: Pocatello (Transit Depot) -&gt; Boise (Airport)</t>
+          <t>d6 Tue 15:40 St George Shuttle: Saint George (Bluff St Office) -&gt; Salt Lake City (Airport)</t>
         </is>
       </c>
     </row>
@@ -4514,17 +4738,17 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>d7 Wed 08:15 Northwestern Stage Lines</t>
+          <t>d6 Tue 18:00 Salt Lake Express</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Boise (Airport)</t>
+          <t>Salt Lake City (Airport)</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Pasco Bus Stop</t>
+          <t>Pocatello (Transit Depot)</t>
         </is>
       </c>
       <c r="E21" s="3" t="n">
@@ -4532,7 +4756,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>d7 Wed 10:30 Greyhound-us: Boise (Chevron) -&gt; Pasco Bus Stop</t>
+          <t>d6 Tue 18:09 Utah Transit Authority: Airport Station -&gt; Gallivan Plaza Station</t>
         </is>
       </c>
     </row>
@@ -4542,25 +4766,25 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>d7 Wed 14:40 FlixBus-us</t>
+          <t>d7 Wed 03:40 Salt Lake Express</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Pasco Bus Stop</t>
+          <t>Pocatello (Transit Depot)</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Spokane Station</t>
-        </is>
-      </c>
-      <c r="E22" s="4" t="n">
-        <v>18.5</v>
+          <t>Boise (Airport)</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="n">
+        <v>24</v>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>d7 Wed 15:00 Northwestern Stage Lines: Pasco Bus Stop -&gt; Spokane</t>
+          <t>d7 Wed 13:25 Salt Lake Express: Pocatello (Transit Depot) -&gt; Boise (Airport)</t>
         </is>
       </c>
     </row>
@@ -4570,25 +4794,25 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>d7 Wed 17:10 Jefferson Lines</t>
+          <t>d7 Wed 08:15 Northwestern Stage Lines</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Spokane</t>
+          <t>Boise (Airport)</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Billings</t>
-        </is>
-      </c>
-      <c r="E23" s="2" t="n">
-        <v>24</v>
+          <t>Pasco Bus Stop</t>
+        </is>
+      </c>
+      <c r="E23" s="3" t="n">
+        <v>0</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>d8 Thu 17:10 Jefferson Lines: Spokane -&gt; Billings</t>
+          <t>d7 Wed 09:02 Valley Regional Transit: Boise Airport -&gt; N Orchard St &amp; W Morris Hill Rd SEC</t>
         </is>
       </c>
     </row>
@@ -4598,25 +4822,25 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>d8 Thu 04:30 Jefferson Lines</t>
+          <t>d7 Wed 14:40 FlixBus-us</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Billings</t>
+          <t>Pasco Bus Stop</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Buffalo</t>
-        </is>
-      </c>
-      <c r="E24" s="2" t="n">
-        <v>24</v>
+          <t>Spokane Station</t>
+        </is>
+      </c>
+      <c r="E24" s="4" t="n">
+        <v>18.5</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>d9 Fri 04:30 Jefferson Lines: Billings -&gt; Buffalo</t>
+          <t>d7 Wed 15:00 Northwestern Stage Lines: Pasco Bus Stop -&gt; Spokane</t>
         </is>
       </c>
     </row>
@@ -4626,17 +4850,17 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>d8 Thu 07:20 Express Arrow</t>
+          <t>d7 Wed 17:10 Jefferson Lines</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Buffalo</t>
+          <t>Spokane</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Denver</t>
+          <t>Billings</t>
         </is>
       </c>
       <c r="E25" s="2" t="n">
@@ -4644,7 +4868,7 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>d9 Fri 07:20 Express Arrow: Buffalo -&gt; Denver</t>
+          <t>d8 Thu 17:10 Jefferson Lines: Spokane -&gt; Billings</t>
         </is>
       </c>
     </row>
@@ -4654,17 +4878,17 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>d8 Thu 18:59 Amtrak</t>
+          <t>d8 Thu 04:30 Jefferson Lines</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Denver</t>
+          <t>Billings</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Omaha Amtrak Station</t>
+          <t>Buffalo</t>
         </is>
       </c>
       <c r="E26" s="2" t="n">
@@ -4672,7 +4896,7 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>d9 Fri 09:25 Express Arrow: Denver -&gt; Omaha</t>
+          <t>d9 Fri 04:30 Jefferson Lines: Billings -&gt; Buffalo</t>
         </is>
       </c>
     </row>
@@ -4682,17 +4906,17 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>d9 Fri 06:15 Jefferson Lines</t>
+          <t>d8 Thu 07:20 Express Arrow</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Omaha</t>
+          <t>Buffalo</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Sioux Falls</t>
+          <t>Denver</t>
         </is>
       </c>
       <c r="E27" s="2" t="n">
@@ -4700,7 +4924,7 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>d10 Sat 06:15 Jefferson Lines: Omaha -&gt; Sioux Falls</t>
+          <t>d9 Fri 07:20 Express Arrow: Buffalo -&gt; Denver</t>
         </is>
       </c>
     </row>
@@ -4710,17 +4934,17 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>d9 Fri 10:00 Jefferson Lines</t>
+          <t>d8 Thu 18:59 Amtrak</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Sioux Falls</t>
+          <t>Denver</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Fargo</t>
+          <t>Omaha Amtrak Station</t>
         </is>
       </c>
       <c r="E28" s="2" t="n">
@@ -4728,7 +4952,7 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>d9 Fri 10:30 Jefferson Lines: Sioux Falls -&gt; Minneapolis</t>
+          <t>d9 Fri 09:25 Express Arrow: Denver -&gt; Omaha</t>
         </is>
       </c>
     </row>
@@ -4738,25 +4962,25 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>d9 Fri 16:40 Jefferson Lines</t>
+          <t>d9 Fri 06:15 Jefferson Lines</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Fargo</t>
+          <t>Omaha</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Minneapolis</t>
-        </is>
-      </c>
-      <c r="E29" s="4" t="n">
-        <v>18.5</v>
+          <t>Sioux Falls</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="n">
+        <v>24</v>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>d9 Fri 17:45 MATBUS: MATBUS - 222 4th St. N -&gt; Shelter 139 (US Bank)</t>
+          <t>d10 Sat 06:15 Jefferson Lines: Omaha -&gt; Sioux Falls</t>
         </is>
       </c>
     </row>
@@ -4766,25 +4990,25 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>d10 Sat 00:15 Greyhound-us</t>
+          <t>d9 Fri 10:00 Jefferson Lines</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Minneapolis Bus Station</t>
+          <t>Sioux Falls</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Chicago Bus Station</t>
-        </is>
-      </c>
-      <c r="E30" s="4" t="n">
-        <v>18.5</v>
+          <t>Fargo</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="n">
+        <v>24</v>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>d10 Sat 07:45 FlixBus-us: Minneapolis Bus Station -&gt; Madison (Madison Campus WI)</t>
+          <t>d10 Sat 10:00 Jefferson Lines: Sioux Falls -&gt; Fargo</t>
         </is>
       </c>
     </row>
@@ -4794,25 +5018,25 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>d10 Sat 09:05 Barons Bus Lines</t>
+          <t>d9 Fri 16:40 Jefferson Lines</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Chicago</t>
+          <t>Fargo</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Toledo (Amtrak)</t>
-        </is>
-      </c>
-      <c r="E31" s="3" t="n">
-        <v>0</v>
+          <t>Minneapolis</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="n">
+        <v>24</v>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>d10 Sat 09:13 Chicago Transit Authority: Jefferson &amp; Harrison -&gt; Randolph &amp; Michigan</t>
+          <t>d10 Sat 10:35 Jefferson Lines: Fargo -&gt; Brainerd</t>
         </is>
       </c>
     </row>
@@ -4822,25 +5046,25 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>d10 Sat 15:35 Greyhound-us</t>
+          <t>d10 Sat 00:15 Greyhound-us</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Toledo Bus Stop</t>
+          <t>Minneapolis Bus Station</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Detroit Bus Station</t>
-        </is>
-      </c>
-      <c r="E32" s="3" t="n">
-        <v>0</v>
+          <t>Chicago Bus Station</t>
+        </is>
+      </c>
+      <c r="E32" s="4" t="n">
+        <v>18.5</v>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>d10 Sat 16:55 Greyhound-us: Toledo Bus Stop -&gt; Detroit Bus Station</t>
+          <t>d10 Sat 07:45 FlixBus-us: Minneapolis Bus Station -&gt; Madison (Madison Campus WI)</t>
         </is>
       </c>
     </row>
@@ -4850,17 +5074,17 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>d10 Sat 19:55 Greyhound-us</t>
+          <t>d10 Sat 09:05 Barons Bus Lines</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Detroit Bus Station</t>
+          <t>Chicago</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Huntington Bus Stop</t>
+          <t>Toledo (Amtrak)</t>
         </is>
       </c>
       <c r="E33" s="4" t="n">
@@ -4868,7 +5092,63 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>d10 Sat 21:30 Amtrak Chartered Vehicle: Detroit -&gt; Toledo</t>
+          <t>d10 Sat 09:13 Chicago Transit Authority: Jefferson &amp; Harrison -&gt; Randolph &amp; Michigan</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>32</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>d10 Sat 15:35 Greyhound-us</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Toledo Bus Stop</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Detroit Bus Station</t>
+        </is>
+      </c>
+      <c r="E34" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>d10 Sat 16:55 Greyhound-us: Toledo Bus Stop -&gt; Detroit Bus Station</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>33</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>d10 Sat 19:55 Greyhound-us</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Detroit Bus Station</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Huntington Bus Stop</t>
+        </is>
+      </c>
+      <c r="E35" s="4" t="n">
+        <v>16.4</v>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>d10 Sat 20:25 Detroit Department of Transportation: Rosa Parks Transit Center - Bay 15 -&gt; Woodward &amp; Baltimore</t>
         </is>
       </c>
     </row>
@@ -4883,7 +5163,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F32"/>
+  <dimension ref="A1:F35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -4897,7 +5177,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Record-Omnibus: 238.83 h from the first bus (search variant of the record: Omnibus KC 13:01 -&gt; Tucumcari). Miss each ride by one minute and replay the rest.</t>
+          <t>Record-Omnibus: 238.83 h from the first bus. Miss each ride by one minute and replay the rest.</t>
         </is>
       </c>
     </row>
@@ -4957,7 +5237,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>d1 Thu 06:40 Dartmouth Coach: Hanover (Hanover Inn) -&gt; Boston South Station</t>
+          <t>d1 Thu 06:01 Advance Transit: Hartford Town Hall, Opp. -&gt; Hanover Inn</t>
         </is>
       </c>
     </row>
@@ -4985,7 +5265,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>d1 Thu 08:50 Amtrak: Boston -&gt; Portland</t>
+          <t>d1 Thu 08:10 Peter Pan (BZ): Boston (South Station) -&gt; Boston (Logan Airport)</t>
         </is>
       </c>
     </row>
@@ -5125,7 +5405,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>wait 1 day(s) and catch the same bus, then continue</t>
+          <t>d2 Fri 21:05 Greyhound-us: Tallahassee (CK Steele Bus Plaza) -&gt; Orlando Bus Station</t>
         </is>
       </c>
     </row>
@@ -5173,7 +5453,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Kansas City 47Th St Transit Center</t>
+          <t>Kansas City Bus Station</t>
         </is>
       </c>
       <c r="E11" s="3" t="n">
@@ -5191,25 +5471,25 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>d4 Sun 13:01 Omnibus Express</t>
+          <t>d4 Sun 05:20 Jefferson Lines</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Kansas City</t>
+          <t>Kansas City Bus Station</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Tucumcari</t>
-        </is>
-      </c>
-      <c r="E12" s="2" t="n">
-        <v>24</v>
+          <t>Tulsa</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="n">
+        <v>0</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>d4 Sun 16:05 Amtrak: Kansas City -&gt; St. Louis</t>
+          <t>d4 Sun 06:15 Greyhound-us: Kansas City Bus Station -&gt; Oklahoma City Bus Station</t>
         </is>
       </c>
     </row>
@@ -5219,12 +5499,12 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>d5 Mon 01:55 Greyhound-us</t>
+          <t>d4 Sun 16:45 Greyhound-us</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Tucumcari (McDonald's)</t>
+          <t>Tulsa Bus Station</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -5237,7 +5517,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>d5 Mon 02:10 Greyhound-us: Tucumcari (McDonald's) -&gt; Amarillo Multimodal Transfer Sta</t>
+          <t>d4 Sun 23:45 Greyhound-us: Tulsa Bus Station -&gt; Springfield CU Transit Center</t>
         </is>
       </c>
     </row>
@@ -5285,7 +5565,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Las Vegas Strip (Las Vegas Blvd)</t>
+          <t>Las Vegas Downtown (1st St)</t>
         </is>
       </c>
       <c r="E15" s="2" t="n">
@@ -5303,17 +5583,17 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>d6 Tue 06:10 Salt Lake Express</t>
+          <t xml:space="preserve">d6 Tue 01:42 Regional Transportation Commission of Southern Nevada </t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Las Vegas (South Strip Transit)</t>
+          <t>Bonneville Transit Center Bay 24</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Saint George (Bluff St Office)</t>
+          <t>EB Wellness before Willow</t>
         </is>
       </c>
       <c r="E16" s="3" t="n">
@@ -5321,7 +5601,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>d6 Tue 06:22 Regional Transportation Commission of Southern Nevada : South Strip Transit Terminal Bay 18 -&gt; Harry Reid Intl Airport Zero Level</t>
+          <t>d6 Tue 02:04 Regional Transportation Commission of Southern Nevada : EB Bonneville after Grand Central -&gt; Harry Reid Intl Airport Zero Level</t>
         </is>
       </c>
     </row>
@@ -5331,17 +5611,17 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>d6 Tue 10:00 Salt Lake Express</t>
+          <t xml:space="preserve">d6 Tue 02:00 Regional Transportation Commission of Southern Nevada </t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Saint George (Bluff St Office)</t>
+          <t>EB Wellness before Willow</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Salt Lake City (Airport)</t>
+          <t>Harry Reid Intl Airport Zero Level</t>
         </is>
       </c>
       <c r="E17" s="3" t="n">
@@ -5349,7 +5629,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>d6 Tue 16:05 Salt Lake Express: Saint George (Shop) -&gt; Salt Lake City (Airport)</t>
+          <t>d6 Tue 02:30 Regional Transportation Commission of Southern Nevada : EB Wellness before Willow -&gt; Harry Reid Intl Airport Zero Level</t>
         </is>
       </c>
     </row>
@@ -5359,17 +5639,17 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>d6 Tue 16:00 Salt Lake Express</t>
+          <t>d6 Tue 06:00 St George Shuttle</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Salt Lake City (Airport)</t>
+          <t>Las Vegas (Airport)</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Pocatello (Transit Depot)</t>
+          <t>Saint George (Bluff St Office)</t>
         </is>
       </c>
       <c r="E18" s="3" t="n">
@@ -5377,7 +5657,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>d6 Tue 16:09 Utah Transit Authority: Airport Station -&gt; North Temple Bridge/Guadalupe</t>
+          <t>d6 Tue 06:30 Salt Lake Express: Las Vegas (Airport) -&gt; Saint George (Bluff St Office)</t>
         </is>
       </c>
     </row>
@@ -5387,25 +5667,25 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>d7 Wed 03:40 Salt Lake Express</t>
+          <t>d6 Tue 09:30 St George Shuttle</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Pocatello (Transit Depot)</t>
+          <t>Saint George (Bluff St Office)</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Boise (Airport)</t>
-        </is>
-      </c>
-      <c r="E19" s="2" t="n">
-        <v>24</v>
+          <t>Orem Central Station (St George Shuttle)</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="n">
+        <v>0</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>d7 Wed 13:25 Salt Lake Express: Pocatello (Transit Depot) -&gt; Boise (Airport)</t>
+          <t>d6 Tue 10:00 Salt Lake Express: Saint George (Bluff St Office) -&gt; Salt Lake City (Airport)</t>
         </is>
       </c>
     </row>
@@ -5415,17 +5695,17 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>d7 Wed 08:15 Northwestern Stage Lines</t>
+          <t>d6 Tue 13:54 Utah Transit Authority</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Boise (Airport)</t>
+          <t>Orem Central Station</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Pasco Bus Stop</t>
+          <t>Salt Lake Central Station</t>
         </is>
       </c>
       <c r="E20" s="3" t="n">
@@ -5433,7 +5713,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>d7 Wed 10:30 Greyhound-us: Boise (Chevron) -&gt; Pasco Bus Stop</t>
+          <t>d6 Tue 14:03 Utah Transit Authority: Orem Central Station -&gt; Provo Central Station</t>
         </is>
       </c>
     </row>
@@ -5443,17 +5723,17 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>d7 Wed 14:40 FlixBus-us</t>
+          <t>d6 Tue 15:15 Salt Lake Express</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Pasco Bus Stop</t>
+          <t>Salt Lake City (Transit Center)</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Spokane Station</t>
+          <t>Pocatello (Transit Depot)</t>
         </is>
       </c>
       <c r="E21" s="3" t="n">
@@ -5461,7 +5741,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>d7 Wed 15:00 Northwestern Stage Lines: Pasco Bus Stop -&gt; Spokane</t>
+          <t>d6 Tue 15:22 Utah Transit Authority: Salt Lake Central Station (Bay A) -&gt; 200 S / 200 W (EB)</t>
         </is>
       </c>
     </row>
@@ -5471,17 +5751,17 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>d7 Wed 17:10 Jefferson Lines</t>
+          <t>d7 Wed 03:40 Salt Lake Express</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Spokane</t>
+          <t>Pocatello (Transit Depot)</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Billings</t>
+          <t>Boise (Airport)</t>
         </is>
       </c>
       <c r="E22" s="2" t="n">
@@ -5489,7 +5769,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>d8 Thu 17:10 Jefferson Lines: Spokane -&gt; Billings</t>
+          <t>d7 Wed 13:25 Salt Lake Express: Pocatello (Transit Depot) -&gt; Boise (Airport)</t>
         </is>
       </c>
     </row>
@@ -5499,25 +5779,25 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>d8 Thu 04:30 Jefferson Lines</t>
+          <t>d7 Wed 08:15 Northwestern Stage Lines</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Billings</t>
+          <t>Boise (Airport)</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Buffalo</t>
-        </is>
-      </c>
-      <c r="E23" s="2" t="n">
-        <v>24</v>
+          <t>Pasco Bus Stop</t>
+        </is>
+      </c>
+      <c r="E23" s="3" t="n">
+        <v>0</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>d9 Fri 04:30 Jefferson Lines: Billings -&gt; Buffalo</t>
+          <t>d7 Wed 09:02 Valley Regional Transit: Boise Airport -&gt; N Orchard St &amp; W Morris Hill Rd SEC</t>
         </is>
       </c>
     </row>
@@ -5527,25 +5807,25 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>d8 Thu 07:20 Express Arrow</t>
+          <t>d7 Wed 14:40 FlixBus-us</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Buffalo</t>
+          <t>Pasco Bus Stop</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Denver</t>
-        </is>
-      </c>
-      <c r="E24" s="2" t="n">
-        <v>24</v>
+          <t>Spokane Station</t>
+        </is>
+      </c>
+      <c r="E24" s="3" t="n">
+        <v>0</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>d9 Fri 07:20 Express Arrow: Buffalo -&gt; Denver</t>
+          <t>d7 Wed 15:00 Northwestern Stage Lines: Pasco Bus Stop -&gt; Spokane</t>
         </is>
       </c>
     </row>
@@ -5555,17 +5835,17 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>d8 Thu 18:59 Amtrak</t>
+          <t>d7 Wed 17:10 Jefferson Lines</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Denver</t>
+          <t>Spokane</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Omaha Amtrak Station</t>
+          <t>Billings</t>
         </is>
       </c>
       <c r="E25" s="2" t="n">
@@ -5573,7 +5853,7 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>d9 Fri 09:25 Express Arrow: Denver -&gt; Omaha</t>
+          <t>d8 Thu 17:10 Jefferson Lines: Spokane -&gt; Billings</t>
         </is>
       </c>
     </row>
@@ -5583,17 +5863,17 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>d9 Fri 06:15 Jefferson Lines</t>
+          <t>d8 Thu 04:30 Jefferson Lines</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Omaha</t>
+          <t>Billings</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Sioux Falls</t>
+          <t>Buffalo</t>
         </is>
       </c>
       <c r="E26" s="2" t="n">
@@ -5601,7 +5881,7 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>d10 Sat 06:15 Jefferson Lines: Omaha -&gt; Sioux Falls</t>
+          <t>d9 Fri 04:30 Jefferson Lines: Billings -&gt; Buffalo</t>
         </is>
       </c>
     </row>
@@ -5611,17 +5891,17 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>d9 Fri 10:00 Jefferson Lines</t>
+          <t>d8 Thu 07:20 Express Arrow</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Sioux Falls</t>
+          <t>Buffalo</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Fargo</t>
+          <t>Denver</t>
         </is>
       </c>
       <c r="E27" s="2" t="n">
@@ -5629,7 +5909,7 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>d9 Fri 10:30 Jefferson Lines: Sioux Falls -&gt; Minneapolis</t>
+          <t>d9 Fri 07:20 Express Arrow: Buffalo -&gt; Denver</t>
         </is>
       </c>
     </row>
@@ -5639,25 +5919,25 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>d9 Fri 16:40 Jefferson Lines</t>
+          <t>d8 Thu 18:59 Amtrak</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Fargo</t>
+          <t>Denver</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Minneapolis</t>
-        </is>
-      </c>
-      <c r="E28" s="4" t="n">
-        <v>18.5</v>
+          <t>Omaha Amtrak Station</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="n">
+        <v>24</v>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>d10 Sat 03:29 Amtrak: Fargo Amtrak Station -&gt; St. Paul-Minneapolis</t>
+          <t>d9 Fri 09:25 Express Arrow: Denver -&gt; Omaha</t>
         </is>
       </c>
     </row>
@@ -5667,25 +5947,25 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>d10 Sat 00:15 Greyhound-us</t>
+          <t>d9 Fri 06:15 Jefferson Lines</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Minneapolis Bus Station</t>
+          <t>Omaha</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Chicago Bus Station</t>
-        </is>
-      </c>
-      <c r="E29" s="4" t="n">
-        <v>18.5</v>
+          <t>Sioux Falls</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="n">
+        <v>24</v>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>d10 Sat 01:29 Metro Transit: Snelling &amp; Dayton Station -&gt; Marshall &amp; Fairview Station</t>
+          <t>d10 Sat 06:15 Jefferson Lines: Omaha -&gt; Sioux Falls</t>
         </is>
       </c>
     </row>
@@ -5695,25 +5975,25 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>d10 Sat 09:05 Barons Bus Lines</t>
+          <t>d9 Fri 10:00 Jefferson Lines</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Chicago</t>
+          <t>Sioux Falls</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Toledo (Amtrak)</t>
-        </is>
-      </c>
-      <c r="E30" s="4" t="n">
-        <v>18.5</v>
+          <t>Fargo</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="n">
+        <v>24</v>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>d10 Sat 12:25 FlixBus-us: Chicago Bus Station -&gt; Toledo Bus Stop</t>
+          <t>d9 Fri 10:30 Jefferson Lines: Sioux Falls -&gt; Minneapolis</t>
         </is>
       </c>
     </row>
@@ -5723,25 +6003,25 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>d10 Sat 15:35 Greyhound-us</t>
+          <t>d9 Fri 16:40 Jefferson Lines</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Toledo Bus Stop</t>
+          <t>Fargo</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Detroit Bus Station</t>
-        </is>
-      </c>
-      <c r="E31" s="3" t="n">
-        <v>0</v>
+          <t>Minneapolis</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="n">
+        <v>24</v>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>d10 Sat 16:55 Greyhound-us: Toledo Bus Stop -&gt; Detroit Bus Station</t>
+          <t>d10 Sat 10:35 Jefferson Lines: Fargo -&gt; Brainerd</t>
         </is>
       </c>
     </row>
@@ -5751,17 +6031,17 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>d10 Sat 19:55 Greyhound-us</t>
+          <t>d10 Sat 00:15 Greyhound-us</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Detroit Bus Station</t>
+          <t>Minneapolis Bus Station</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Huntington Bus Stop</t>
+          <t>Chicago Bus Station</t>
         </is>
       </c>
       <c r="E32" s="4" t="n">
@@ -5769,7 +6049,91 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>d10 Sat 21:30 Amtrak Chartered Vehicle: Detroit -&gt; Toledo</t>
+          <t>d10 Sat 07:45 FlixBus-us: Minneapolis Bus Station -&gt; Madison (Madison Campus WI)</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>31</v>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>d10 Sat 09:05 Barons Bus Lines</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Chicago</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Toledo (Amtrak)</t>
+        </is>
+      </c>
+      <c r="E33" s="4" t="n">
+        <v>16.4</v>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>d10 Sat 09:13 Chicago Transit Authority: Jefferson &amp; Harrison -&gt; Randolph &amp; Michigan</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>32</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>d10 Sat 15:35 Greyhound-us</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Toledo Bus Stop</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Detroit Bus Station</t>
+        </is>
+      </c>
+      <c r="E34" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>d10 Sat 16:55 Greyhound-us: Toledo Bus Stop -&gt; Detroit Bus Station</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>33</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>d10 Sat 19:55 Greyhound-us</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Detroit Bus Station</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Huntington Bus Stop</t>
+        </is>
+      </c>
+      <c r="E35" s="4" t="n">
+        <v>16.4</v>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>d10 Sat 20:25 Detroit Department of Transportation: Rosa Parks Transit Center - Bay 15 -&gt; Woodward &amp; Baltimore</t>
         </is>
       </c>
     </row>

</xml_diff>